<commit_message>
Clean up repo and push current changes
_R_code is the main code folder now. There is also a data folder with necessary files. Also trying gitattributes for data uploading?
</commit_message>
<xml_diff>
--- a/manuscript/BANTER_Pseudorca-AllTablesxlsx.xlsx
+++ b/manuscript/BANTER_Pseudorca-AllTablesxlsx.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jennifer.McCullough\Documents\GitHub\BANTER_Pseudorca\manuscript\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yvonne.barkley\Github\BANTER_Pseudorca\manuscript\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B6CC7E0-0448-4CB9-A710-E09D139487D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66D9931E-3541-4DC1-BFF3-EEC28517D345}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Threshold_Table" sheetId="4" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="205" uniqueCount="126">
   <si>
     <t>Survey Year</t>
   </si>
@@ -177,9 +177,6 @@
     <t>SE-18-03</t>
   </si>
   <si>
-    <t>SE-17-06; LR-17-05</t>
-  </si>
-  <si>
     <t>SE-16-04</t>
   </si>
   <si>
@@ -406,6 +403,21 @@
   </si>
   <si>
     <t>12 (0)</t>
+  </si>
+  <si>
+    <t>Visually-Verified Acoustic Pseudorca Events</t>
+  </si>
+  <si>
+    <t>Visually-Verified Acoustic Other Events</t>
+  </si>
+  <si>
+    <t>8; 1</t>
+  </si>
+  <si>
+    <t>LR-17-05; SE-17-06</t>
+  </si>
+  <si>
+    <t>10; 11</t>
   </si>
 </sst>
 </file>
@@ -460,7 +472,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -470,6 +482,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -740,7 +758,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -785,9 +803,6 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
@@ -846,6 +861,15 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1129,388 +1153,388 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{16B82A36-BAB4-4DA2-945D-9C525C938092}">
   <dimension ref="A1:Q8"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="16.28515625" style="24" customWidth="1"/>
-    <col min="2" max="2" width="11.42578125" style="25" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="6.85546875" style="25" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="7.85546875" style="25" customWidth="1"/>
-    <col min="6" max="8" width="6.85546875" style="25" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="7.85546875" style="25" bestFit="1" customWidth="1"/>
-    <col min="10" max="12" width="5.85546875" style="25" bestFit="1" customWidth="1"/>
-    <col min="13" max="14" width="7.85546875" style="25" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="8.5703125" style="25" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="6.85546875" style="25" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="7.85546875" style="25" bestFit="1" customWidth="1"/>
-    <col min="18" max="16384" width="9.140625" style="25"/>
+    <col min="1" max="1" width="16.33203125" style="23" customWidth="1"/>
+    <col min="2" max="2" width="11.44140625" style="24" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="6.88671875" style="24" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="7.88671875" style="24" customWidth="1"/>
+    <col min="6" max="8" width="6.88671875" style="24" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="7.88671875" style="24" bestFit="1" customWidth="1"/>
+    <col min="10" max="12" width="5.88671875" style="24" bestFit="1" customWidth="1"/>
+    <col min="13" max="14" width="7.88671875" style="24" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="8.5546875" style="24" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="6.88671875" style="24" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="7.88671875" style="24" bestFit="1" customWidth="1"/>
+    <col min="18" max="16384" width="9.109375" style="24"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="27"/>
-      <c r="B1" s="37" t="s">
+    <row r="1" spans="1:17" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="26"/>
+      <c r="B1" s="36" t="s">
+        <v>61</v>
+      </c>
+      <c r="C1" s="36"/>
+      <c r="D1" s="36"/>
+      <c r="E1" s="36"/>
+      <c r="F1" s="27"/>
+      <c r="G1" s="27"/>
+      <c r="H1" s="27"/>
+      <c r="I1" s="27"/>
+      <c r="J1" s="27"/>
+      <c r="K1" s="34"/>
+      <c r="L1" s="34"/>
+      <c r="M1" s="34"/>
+      <c r="N1" s="34"/>
+      <c r="O1" s="37" t="s">
         <v>62</v>
       </c>
-      <c r="C1" s="37"/>
-      <c r="D1" s="37"/>
-      <c r="E1" s="37"/>
-      <c r="F1" s="28"/>
-      <c r="G1" s="28"/>
-      <c r="H1" s="28"/>
-      <c r="I1" s="28"/>
-      <c r="J1" s="28"/>
-      <c r="K1" s="35"/>
-      <c r="L1" s="35"/>
-      <c r="M1" s="35"/>
-      <c r="N1" s="35"/>
-      <c r="O1" s="38" t="s">
+      <c r="P1" s="34"/>
+      <c r="Q1" s="35"/>
+    </row>
+    <row r="2" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A2" s="38" t="s">
         <v>63</v>
       </c>
-      <c r="P1" s="35"/>
-      <c r="Q1" s="36"/>
-    </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A2" s="39" t="s">
+      <c r="B2" s="26">
+        <v>2017</v>
+      </c>
+      <c r="C2" s="27"/>
+      <c r="D2" s="27"/>
+      <c r="E2" s="28"/>
+      <c r="F2" s="26">
+        <v>2023</v>
+      </c>
+      <c r="G2" s="27"/>
+      <c r="H2" s="27"/>
+      <c r="I2" s="28"/>
+      <c r="J2" s="26">
+        <v>2024</v>
+      </c>
+      <c r="K2" s="34"/>
+      <c r="L2" s="34"/>
+      <c r="M2" s="35"/>
+      <c r="N2" s="26" t="s">
+        <v>50</v>
+      </c>
+      <c r="O2" s="34"/>
+      <c r="P2" s="34"/>
+      <c r="Q2" s="35"/>
+    </row>
+    <row r="3" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A3" s="39"/>
+      <c r="B3" s="29" t="s">
         <v>64</v>
       </c>
-      <c r="B2" s="27">
-        <v>2017</v>
-      </c>
-      <c r="C2" s="28"/>
-      <c r="D2" s="28"/>
-      <c r="E2" s="29"/>
-      <c r="F2" s="27">
-        <v>2023</v>
-      </c>
-      <c r="G2" s="28"/>
-      <c r="H2" s="28"/>
-      <c r="I2" s="29"/>
-      <c r="J2" s="27">
-        <v>2024</v>
-      </c>
-      <c r="K2" s="35"/>
-      <c r="L2" s="35"/>
-      <c r="M2" s="36"/>
-      <c r="N2" s="27" t="s">
-        <v>51</v>
-      </c>
-      <c r="O2" s="35"/>
-      <c r="P2" s="35"/>
-      <c r="Q2" s="36"/>
-    </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A3" s="40"/>
-      <c r="B3" s="30" t="s">
+      <c r="C3" s="25" t="s">
         <v>65</v>
       </c>
-      <c r="C3" s="26" t="s">
+      <c r="D3" s="25" t="s">
         <v>66</v>
       </c>
-      <c r="D3" s="26" t="s">
+      <c r="E3" s="30" t="s">
         <v>67</v>
       </c>
-      <c r="E3" s="31" t="s">
+      <c r="F3" s="29" t="s">
         <v>68</v>
       </c>
-      <c r="F3" s="30" t="s">
+      <c r="G3" s="25" t="s">
+        <v>65</v>
+      </c>
+      <c r="H3" s="25" t="s">
+        <v>66</v>
+      </c>
+      <c r="I3" s="30" t="s">
+        <v>67</v>
+      </c>
+      <c r="J3" s="29" t="s">
+        <v>68</v>
+      </c>
+      <c r="K3" s="25" t="s">
+        <v>65</v>
+      </c>
+      <c r="L3" s="25" t="s">
+        <v>66</v>
+      </c>
+      <c r="M3" s="30" t="s">
+        <v>67</v>
+      </c>
+      <c r="N3" s="29" t="s">
+        <v>68</v>
+      </c>
+      <c r="O3" s="25" t="s">
+        <v>65</v>
+      </c>
+      <c r="P3" s="25" t="s">
+        <v>66</v>
+      </c>
+      <c r="Q3" s="30" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="4" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A4" s="40">
+        <v>0.5</v>
+      </c>
+      <c r="B4" s="29" t="s">
         <v>69</v>
       </c>
-      <c r="G3" s="26" t="s">
-        <v>66</v>
-      </c>
-      <c r="H3" s="26" t="s">
-        <v>67</v>
-      </c>
-      <c r="I3" s="31" t="s">
-        <v>68</v>
-      </c>
-      <c r="J3" s="30" t="s">
-        <v>69</v>
-      </c>
-      <c r="K3" s="26" t="s">
-        <v>66</v>
-      </c>
-      <c r="L3" s="26" t="s">
-        <v>67</v>
-      </c>
-      <c r="M3" s="31" t="s">
-        <v>68</v>
-      </c>
-      <c r="N3" s="30" t="s">
-        <v>69</v>
-      </c>
-      <c r="O3" s="26" t="s">
-        <v>66</v>
-      </c>
-      <c r="P3" s="26" t="s">
-        <v>67</v>
-      </c>
-      <c r="Q3" s="31" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A4" s="41">
-        <v>0.5</v>
-      </c>
-      <c r="B4" s="30" t="s">
+      <c r="C4" s="25" t="s">
         <v>70</v>
       </c>
-      <c r="C4" s="26" t="s">
+      <c r="D4" s="25" t="s">
         <v>71</v>
       </c>
-      <c r="D4" s="26" t="s">
+      <c r="E4" s="30" t="s">
         <v>72</v>
       </c>
-      <c r="E4" s="31" t="s">
+      <c r="F4" s="29" t="s">
         <v>73</v>
       </c>
-      <c r="F4" s="30" t="s">
+      <c r="G4" s="25" t="s">
         <v>74</v>
       </c>
-      <c r="G4" s="26" t="s">
+      <c r="H4" s="25" t="s">
         <v>75</v>
       </c>
-      <c r="H4" s="26" t="s">
+      <c r="I4" s="30" t="s">
         <v>76</v>
       </c>
-      <c r="I4" s="31" t="s">
+      <c r="J4" s="29" t="s">
         <v>77</v>
       </c>
-      <c r="J4" s="30" t="s">
+      <c r="K4" s="25" t="s">
         <v>78</v>
       </c>
-      <c r="K4" s="26" t="s">
+      <c r="L4" s="25" t="s">
         <v>79</v>
       </c>
-      <c r="L4" s="26" t="s">
+      <c r="M4" s="30" t="s">
         <v>80</v>
       </c>
-      <c r="M4" s="31" t="s">
+      <c r="N4" s="29" t="s">
         <v>81</v>
       </c>
-      <c r="N4" s="30" t="s">
+      <c r="O4" s="25" t="s">
         <v>82</v>
       </c>
-      <c r="O4" s="26" t="s">
+      <c r="P4" s="25" t="s">
         <v>83</v>
       </c>
-      <c r="P4" s="26" t="s">
+      <c r="Q4" s="30" t="s">
         <v>84</v>
       </c>
-      <c r="Q4" s="31" t="s">
+    </row>
+    <row r="5" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A5" s="40">
+        <v>0.6</v>
+      </c>
+      <c r="B5" s="29" t="s">
         <v>85</v>
       </c>
-    </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A5" s="41">
-        <v>0.6</v>
-      </c>
-      <c r="B5" s="30" t="s">
+      <c r="C5" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="C5" s="26" t="s">
+      <c r="D5" s="25" t="s">
         <v>87</v>
       </c>
-      <c r="D5" s="26" t="s">
+      <c r="E5" s="30" t="s">
+        <v>72</v>
+      </c>
+      <c r="F5" s="29" t="s">
         <v>88</v>
       </c>
-      <c r="E5" s="31" t="s">
-        <v>73</v>
-      </c>
-      <c r="F5" s="30" t="s">
+      <c r="G5" s="25" t="s">
         <v>89</v>
       </c>
-      <c r="G5" s="26" t="s">
+      <c r="H5" s="25" t="s">
         <v>90</v>
       </c>
-      <c r="H5" s="26" t="s">
+      <c r="I5" s="30" t="s">
+        <v>80</v>
+      </c>
+      <c r="J5" s="29" t="s">
         <v>91</v>
       </c>
-      <c r="I5" s="31" t="s">
-        <v>81</v>
-      </c>
-      <c r="J5" s="30" t="s">
+      <c r="K5" s="25" t="s">
         <v>92</v>
       </c>
-      <c r="K5" s="26" t="s">
+      <c r="L5" s="25" t="s">
+        <v>91</v>
+      </c>
+      <c r="M5" s="30" t="s">
+        <v>92</v>
+      </c>
+      <c r="N5" s="29" t="s">
+        <v>83</v>
+      </c>
+      <c r="O5" s="25" t="s">
         <v>93</v>
       </c>
-      <c r="L5" s="26" t="s">
-        <v>92</v>
-      </c>
-      <c r="M5" s="31" t="s">
-        <v>93</v>
-      </c>
-      <c r="N5" s="30" t="s">
-        <v>84</v>
-      </c>
-      <c r="O5" s="26" t="s">
+      <c r="P5" s="25" t="s">
         <v>94</v>
       </c>
-      <c r="P5" s="26" t="s">
+      <c r="Q5" s="30" t="s">
         <v>95</v>
       </c>
-      <c r="Q5" s="31" t="s">
+    </row>
+    <row r="6" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A6" s="40">
+        <v>0.7</v>
+      </c>
+      <c r="B6" s="29" t="s">
         <v>96</v>
       </c>
-    </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A6" s="41">
-        <v>0.7</v>
-      </c>
-      <c r="B6" s="30" t="s">
+      <c r="C6" s="25" t="s">
         <v>97</v>
       </c>
-      <c r="C6" s="26" t="s">
+      <c r="D6" s="25" t="s">
         <v>98</v>
       </c>
-      <c r="D6" s="26" t="s">
+      <c r="E6" s="30" t="s">
         <v>99</v>
       </c>
-      <c r="E6" s="31" t="s">
+      <c r="F6" s="29" t="s">
         <v>100</v>
       </c>
-      <c r="F6" s="30" t="s">
+      <c r="G6" s="25" t="s">
         <v>101</v>
       </c>
-      <c r="G6" s="26" t="s">
+      <c r="H6" s="25" t="s">
         <v>102</v>
       </c>
-      <c r="H6" s="26" t="s">
+      <c r="I6" s="30" t="s">
         <v>103</v>
       </c>
-      <c r="I6" s="31" t="s">
+      <c r="J6" s="29" t="s">
         <v>104</v>
       </c>
-      <c r="J6" s="30" t="s">
+      <c r="K6" s="25" t="s">
+        <v>103</v>
+      </c>
+      <c r="L6" s="25" t="s">
+        <v>104</v>
+      </c>
+      <c r="M6" s="30" t="s">
+        <v>103</v>
+      </c>
+      <c r="N6" s="29" t="s">
         <v>105</v>
       </c>
-      <c r="K6" s="26" t="s">
-        <v>104</v>
-      </c>
-      <c r="L6" s="26" t="s">
-        <v>105</v>
-      </c>
-      <c r="M6" s="31" t="s">
-        <v>104</v>
-      </c>
-      <c r="N6" s="30" t="s">
+      <c r="O6" s="25" t="s">
         <v>106</v>
       </c>
-      <c r="O6" s="26" t="s">
+      <c r="P6" s="25" t="s">
         <v>107</v>
       </c>
-      <c r="P6" s="26" t="s">
+      <c r="Q6" s="30" t="s">
         <v>108</v>
       </c>
-      <c r="Q6" s="31" t="s">
+    </row>
+    <row r="7" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A7" s="40">
+        <v>0.8</v>
+      </c>
+      <c r="B7" s="29" t="s">
         <v>109</v>
       </c>
-    </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A7" s="41">
-        <v>0.8</v>
-      </c>
-      <c r="B7" s="30" t="s">
+      <c r="C7" s="25" t="s">
         <v>110</v>
       </c>
-      <c r="C7" s="26" t="s">
+      <c r="D7" s="25" t="s">
+        <v>109</v>
+      </c>
+      <c r="E7" s="30" t="s">
+        <v>110</v>
+      </c>
+      <c r="F7" s="29" t="s">
         <v>111</v>
       </c>
-      <c r="D7" s="26" t="s">
-        <v>110</v>
-      </c>
-      <c r="E7" s="31" t="s">
-        <v>111</v>
-      </c>
-      <c r="F7" s="30" t="s">
+      <c r="G7" s="25" t="s">
         <v>112</v>
       </c>
-      <c r="G7" s="26" t="s">
+      <c r="H7" s="25" t="s">
+        <v>112</v>
+      </c>
+      <c r="I7" s="30" t="s">
         <v>113</v>
       </c>
-      <c r="H7" s="26" t="s">
-        <v>113</v>
-      </c>
-      <c r="I7" s="31" t="s">
+      <c r="J7" s="29" t="s">
         <v>114</v>
       </c>
-      <c r="J7" s="30" t="s">
+      <c r="K7" s="25" t="s">
+        <v>114</v>
+      </c>
+      <c r="L7" s="25" t="s">
+        <v>114</v>
+      </c>
+      <c r="M7" s="30" t="s">
+        <v>114</v>
+      </c>
+      <c r="N7" s="29" t="s">
         <v>115</v>
       </c>
-      <c r="K7" s="26" t="s">
-        <v>115</v>
-      </c>
-      <c r="L7" s="26" t="s">
-        <v>115</v>
-      </c>
-      <c r="M7" s="31" t="s">
-        <v>115</v>
-      </c>
-      <c r="N7" s="30" t="s">
+      <c r="O7" s="25" t="s">
         <v>116</v>
       </c>
-      <c r="O7" s="26" t="s">
+      <c r="P7" s="25" t="s">
         <v>117</v>
       </c>
-      <c r="P7" s="26" t="s">
+      <c r="Q7" s="30" t="s">
         <v>118</v>
       </c>
-      <c r="Q7" s="31" t="s">
+    </row>
+    <row r="8" spans="1:17" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="41">
+        <v>0.9</v>
+      </c>
+      <c r="B8" s="31" t="s">
+        <v>114</v>
+      </c>
+      <c r="C8" s="32" t="s">
+        <v>114</v>
+      </c>
+      <c r="D8" s="32" t="s">
+        <v>114</v>
+      </c>
+      <c r="E8" s="33" t="s">
+        <v>114</v>
+      </c>
+      <c r="F8" s="31" t="s">
         <v>119</v>
       </c>
-    </row>
-    <row r="8" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="42">
-        <v>0.9</v>
-      </c>
-      <c r="B8" s="32" t="s">
-        <v>115</v>
-      </c>
-      <c r="C8" s="33" t="s">
-        <v>115</v>
-      </c>
-      <c r="D8" s="33" t="s">
-        <v>115</v>
-      </c>
-      <c r="E8" s="34" t="s">
-        <v>115</v>
-      </c>
-      <c r="F8" s="32" t="s">
+      <c r="G8" s="32" t="s">
+        <v>119</v>
+      </c>
+      <c r="H8" s="32" t="s">
+        <v>119</v>
+      </c>
+      <c r="I8" s="33" t="s">
+        <v>119</v>
+      </c>
+      <c r="J8" s="31" t="s">
+        <v>119</v>
+      </c>
+      <c r="K8" s="32" t="s">
+        <v>119</v>
+      </c>
+      <c r="L8" s="32" t="s">
+        <v>119</v>
+      </c>
+      <c r="M8" s="33" t="s">
+        <v>119</v>
+      </c>
+      <c r="N8" s="31" t="s">
         <v>120</v>
       </c>
-      <c r="G8" s="33" t="s">
+      <c r="O8" s="32" t="s">
         <v>120</v>
       </c>
-      <c r="H8" s="33" t="s">
+      <c r="P8" s="32" t="s">
         <v>120</v>
       </c>
-      <c r="I8" s="34" t="s">
+      <c r="Q8" s="33" t="s">
         <v>120</v>
-      </c>
-      <c r="J8" s="32" t="s">
-        <v>120</v>
-      </c>
-      <c r="K8" s="33" t="s">
-        <v>120</v>
-      </c>
-      <c r="L8" s="33" t="s">
-        <v>120</v>
-      </c>
-      <c r="M8" s="34" t="s">
-        <v>120</v>
-      </c>
-      <c r="N8" s="32" t="s">
-        <v>121</v>
-      </c>
-      <c r="O8" s="33" t="s">
-        <v>121</v>
-      </c>
-      <c r="P8" s="33" t="s">
-        <v>121</v>
-      </c>
-      <c r="Q8" s="34" t="s">
-        <v>121</v>
       </c>
     </row>
   </sheetData>
@@ -1521,14 +1545,14 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B2:K15"/>
-  <sheetFormatPr defaultColWidth="14.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="B2:M15"/>
+  <sheetFormatPr defaultColWidth="14.33203125" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="10" customWidth="1"/>
-    <col min="3" max="4" width="23.28515625" style="1" customWidth="1"/>
+    <col min="3" max="4" width="23.33203125" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:11" ht="57" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:13" ht="83.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B2" s="12" t="s">
         <v>0</v>
       </c>
@@ -1541,7 +1565,7 @@
       <c r="E2" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="F2" s="12" t="s">
+      <c r="F2" s="43" t="s">
         <v>3</v>
       </c>
       <c r="G2" s="12" t="s">
@@ -1557,10 +1581,16 @@
         <v>18</v>
       </c>
       <c r="K2" s="12" t="s">
+        <v>121</v>
+      </c>
+      <c r="L2" s="12" t="s">
+        <v>122</v>
+      </c>
+      <c r="M2" s="12" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="2:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:13" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B3" s="12">
         <v>2010</v>
       </c>
@@ -1568,7 +1598,7 @@
         <v>5</v>
       </c>
       <c r="D3" s="13" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E3" s="14" t="s">
         <v>11</v>
@@ -1586,9 +1616,13 @@
       <c r="J3" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="K3" s="14"/>
-    </row>
-    <row r="4" spans="2:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K3" s="44" t="s">
+        <v>123</v>
+      </c>
+      <c r="L3" s="2"/>
+      <c r="M3" s="14"/>
+    </row>
+    <row r="4" spans="2:13" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B4" s="12">
         <v>2011</v>
       </c>
@@ -1612,9 +1646,13 @@
       <c r="J4" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="K4" s="14"/>
-    </row>
-    <row r="5" spans="2:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K4" s="44">
+        <v>2</v>
+      </c>
+      <c r="L4" s="2"/>
+      <c r="M4" s="14"/>
+    </row>
+    <row r="5" spans="2:13" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="12">
         <v>2012</v>
       </c>
@@ -1622,7 +1660,7 @@
         <v>10</v>
       </c>
       <c r="D5" s="13" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E5" s="14" t="s">
         <v>11</v>
@@ -1640,9 +1678,13 @@
       <c r="J5" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="K5" s="14"/>
-    </row>
-    <row r="6" spans="2:11" ht="50.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K5" s="44">
+        <v>1</v>
+      </c>
+      <c r="L5" s="2"/>
+      <c r="M5" s="14"/>
+    </row>
+    <row r="6" spans="2:13" ht="50.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6" s="12">
         <v>2013</v>
       </c>
@@ -1650,7 +1692,7 @@
         <v>14</v>
       </c>
       <c r="D6" s="13" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E6" s="14" t="s">
         <v>12</v>
@@ -1668,9 +1710,13 @@
       <c r="J6" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="K6" s="14"/>
-    </row>
-    <row r="7" spans="2:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K6" s="2">
+        <v>2</v>
+      </c>
+      <c r="L6" s="2"/>
+      <c r="M6" s="14"/>
+    </row>
+    <row r="7" spans="2:13" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="12">
         <v>2015</v>
       </c>
@@ -1678,7 +1724,7 @@
         <v>7</v>
       </c>
       <c r="D7" s="13" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E7" s="14" t="s">
         <v>13</v>
@@ -1694,9 +1740,13 @@
       <c r="J7" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="K7" s="14"/>
-    </row>
-    <row r="8" spans="2:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K7" s="2">
+        <v>2</v>
+      </c>
+      <c r="L7" s="2"/>
+      <c r="M7" s="14"/>
+    </row>
+    <row r="8" spans="2:13" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B8" s="12">
         <v>2016</v>
       </c>
@@ -1704,7 +1754,7 @@
         <v>6</v>
       </c>
       <c r="D8" s="13" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E8" s="14" t="s">
         <v>13</v>
@@ -1722,9 +1772,13 @@
       <c r="J8" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="K8" s="14"/>
-    </row>
-    <row r="9" spans="2:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K8" s="2">
+        <v>1</v>
+      </c>
+      <c r="L8" s="2"/>
+      <c r="M8" s="14"/>
+    </row>
+    <row r="9" spans="2:13" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B9" s="12">
         <v>2017</v>
       </c>
@@ -1732,7 +1786,7 @@
         <v>5</v>
       </c>
       <c r="D9" s="13" t="s">
-        <v>45</v>
+        <v>124</v>
       </c>
       <c r="E9" s="14" t="s">
         <v>13</v>
@@ -1750,9 +1804,13 @@
       <c r="J9" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="K9" s="14"/>
-    </row>
-    <row r="10" spans="2:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K9" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="L9" s="2"/>
+      <c r="M9" s="14"/>
+    </row>
+    <row r="10" spans="2:13" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B10" s="12">
         <v>2018</v>
       </c>
@@ -1776,9 +1834,11 @@
       <c r="J10" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="K10" s="14"/>
-    </row>
-    <row r="11" spans="2:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K10" s="2"/>
+      <c r="L10" s="2"/>
+      <c r="M10" s="14"/>
+    </row>
+    <row r="11" spans="2:13" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B11" s="12">
         <v>2019</v>
       </c>
@@ -1802,9 +1862,11 @@
       <c r="J11" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="K11" s="14"/>
-    </row>
-    <row r="12" spans="2:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K11" s="2"/>
+      <c r="L11" s="2"/>
+      <c r="M11" s="14"/>
+    </row>
+    <row r="12" spans="2:13" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B12" s="12">
         <v>2020</v>
       </c>
@@ -1828,9 +1890,13 @@
       <c r="J12" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="K12" s="14"/>
-    </row>
-    <row r="13" spans="2:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K12" s="2">
+        <v>4</v>
+      </c>
+      <c r="L12" s="2"/>
+      <c r="M12" s="14"/>
+    </row>
+    <row r="13" spans="2:13" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B13" s="12">
         <v>2021</v>
       </c>
@@ -1854,9 +1920,13 @@
       <c r="J13" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="K13" s="14"/>
-    </row>
-    <row r="14" spans="2:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K13" s="2">
+        <v>9</v>
+      </c>
+      <c r="L13" s="2"/>
+      <c r="M13" s="14"/>
+    </row>
+    <row r="14" spans="2:13" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B14" s="12">
         <v>2023</v>
       </c>
@@ -1880,9 +1950,11 @@
       <c r="J14" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="K14" s="14"/>
-    </row>
-    <row r="15" spans="2:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K14" s="2"/>
+      <c r="L14" s="2"/>
+      <c r="M14" s="14"/>
+    </row>
+    <row r="15" spans="2:13" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B15" s="12">
         <v>2024</v>
       </c>
@@ -1906,7 +1978,9 @@
       <c r="J15" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="K15" s="14"/>
+      <c r="K15" s="2"/>
+      <c r="L15" s="2"/>
+      <c r="M15" s="14"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1917,16 +1991,16 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{53C3CA73-E650-4EB7-93C1-D459BAC41A38}">
   <dimension ref="A3:L31"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="19.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.85546875" customWidth="1"/>
-    <col min="5" max="5" width="10.42578125" customWidth="1"/>
-    <col min="6" max="12" width="10.28515625" customWidth="1"/>
+    <col min="1" max="1" width="19.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.5546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.88671875" customWidth="1"/>
+    <col min="5" max="5" width="10.44140625" customWidth="1"/>
+    <col min="6" max="12" width="10.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:12" ht="75.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:12" ht="72.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B3" s="18" t="s">
         <v>0</v>
       </c>
@@ -1954,7 +2028,7 @@
       </c>
       <c r="L3" s="15"/>
     </row>
-    <row r="4" spans="2:12" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:12" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="B4" s="17">
         <v>2017</v>
       </c>
@@ -1987,7 +2061,7 @@
         <v>445</v>
       </c>
     </row>
-    <row r="5" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B5" s="17">
         <v>2023</v>
       </c>
@@ -2020,7 +2094,7 @@
         <v>321</v>
       </c>
     </row>
-    <row r="6" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B6" s="19">
         <v>2024</v>
       </c>
@@ -2053,8 +2127,8 @@
         <v>87</v>
       </c>
     </row>
-    <row r="7" spans="2:12" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
-    <row r="9" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:12" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
+    <row r="9" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B9" t="s">
         <v>36</v>
       </c>
@@ -2079,7 +2153,7 @@
         <v>0.75</v>
       </c>
     </row>
-    <row r="12" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B12" t="s">
         <v>35</v>
       </c>
@@ -2088,31 +2162,31 @@
         <v>209</v>
       </c>
     </row>
-    <row r="14" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:12" x14ac:dyDescent="0.3">
       <c r="C14" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A17" s="22" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A17" s="21" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B18" t="s">
+        <v>50</v>
+      </c>
+      <c r="C18" t="s">
         <v>51</v>
       </c>
-      <c r="C18" t="s">
+      <c r="D18" t="s">
         <v>52</v>
       </c>
-      <c r="D18" t="s">
+      <c r="E18" t="s">
         <v>53</v>
       </c>
-      <c r="E18" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B19">
         <v>555</v>
       </c>
@@ -2122,12 +2196,12 @@
       <c r="D19">
         <v>33</v>
       </c>
-      <c r="E19" s="21">
+      <c r="E19" s="20">
         <f>(B19-C19)/B19</f>
         <v>0.80180180180180183</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B20">
         <v>388</v>
       </c>
@@ -2137,12 +2211,12 @@
       <c r="D20">
         <v>14</v>
       </c>
-      <c r="E20" s="21">
+      <c r="E20" s="20">
         <f t="shared" ref="E20:E21" si="2">(B20-C20)/B20</f>
         <v>0.82731958762886593</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B21">
         <v>122</v>
       </c>
@@ -2152,79 +2226,79 @@
       <c r="D21">
         <v>10</v>
       </c>
-      <c r="E21" s="21">
+      <c r="E21" s="20">
         <f t="shared" si="2"/>
         <v>0.71311475409836067</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A22" s="22" t="s">
-        <v>51</v>
-      </c>
-      <c r="B22" s="22">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A22" s="21" t="s">
+        <v>50</v>
+      </c>
+      <c r="B22" s="21">
         <f>SUM(B19:B21)</f>
         <v>1065</v>
       </c>
-      <c r="C22" s="22">
+      <c r="C22" s="21">
         <f>SUM(C19:C21)</f>
         <v>212</v>
       </c>
-      <c r="D22" s="22">
+      <c r="D22" s="21">
         <f>SUM(D19:D21)</f>
         <v>57</v>
       </c>
-      <c r="E22" s="22"/>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E22" s="21"/>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B24">
         <f>1068-755</f>
         <v>313</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B25">
         <f>755-212</f>
         <v>543</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A26" s="22" t="s">
-        <v>57</v>
-      </c>
-      <c r="B26" s="22">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A26" s="21" t="s">
+        <v>56</v>
+      </c>
+      <c r="B26" s="21">
         <f>B24+B25</f>
         <v>856</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A28" s="22" t="s">
-        <v>58</v>
-      </c>
-      <c r="B28" s="23">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A28" s="21" t="s">
+        <v>57</v>
+      </c>
+      <c r="B28" s="22">
         <f>B26/B22</f>
         <v>0.8037558685446009</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A30" s="22" t="s">
-        <v>59</v>
-      </c>
-      <c r="B30" s="21">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A30" s="21" t="s">
+        <v>58</v>
+      </c>
+      <c r="B30" s="20">
         <f>AVERAGE(E19:E21)</f>
         <v>0.78074538117634285</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>60</v>
-      </c>
-      <c r="B31" s="21">
+        <v>59</v>
+      </c>
+      <c r="B31" s="20">
         <f>MEDIAN(E19:E21)</f>
         <v>0.80180180180180183</v>
       </c>
@@ -2238,21 +2312,21 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC43C8DF-330E-4085-938E-0299F38AFB9F}">
   <dimension ref="B3:G13"/>
-  <sheetFormatPr defaultColWidth="21.5703125" defaultRowHeight="26.25" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="21.5546875" defaultRowHeight="26.25" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="10.28515625" customWidth="1"/>
-    <col min="2" max="2" width="10.85546875" customWidth="1"/>
-    <col min="3" max="3" width="13.85546875" customWidth="1"/>
-    <col min="4" max="4" width="12.5703125" customWidth="1"/>
-    <col min="5" max="5" width="11.7109375" customWidth="1"/>
+    <col min="1" max="1" width="10.33203125" customWidth="1"/>
+    <col min="2" max="2" width="10.88671875" customWidth="1"/>
+    <col min="3" max="3" width="13.88671875" customWidth="1"/>
+    <col min="4" max="4" width="12.5546875" customWidth="1"/>
+    <col min="5" max="5" width="11.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:7" ht="26.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C3" s="20"/>
-      <c r="D3" s="20"/>
-      <c r="E3" s="20"/>
-    </row>
-    <row r="4" spans="2:7" ht="56.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:7" ht="26.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="C3" s="42"/>
+      <c r="D3" s="42"/>
+      <c r="E3" s="42"/>
+    </row>
+    <row r="4" spans="2:7" ht="56.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B4" s="4"/>
       <c r="C4" s="7" t="s">
         <v>22</v>
@@ -2264,7 +2338,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="5" spans="2:7" ht="26.25" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:7" ht="26.25" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
       <c r="B5" s="11">
         <v>2017</v>
       </c>
@@ -2286,7 +2360,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="6" spans="2:7" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:7" ht="26.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6" s="6">
         <v>2023</v>
       </c>
@@ -2308,7 +2382,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="7" spans="2:7" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:7" ht="26.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="6">
         <v>2024</v>
       </c>
@@ -2330,37 +2404,37 @@
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="2:7" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:7" ht="26.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B8" s="3"/>
       <c r="C8" s="3"/>
       <c r="D8" s="3"/>
       <c r="E8" s="3"/>
     </row>
-    <row r="9" spans="2:7" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:7" ht="26.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B9" s="3"/>
       <c r="C9" s="3"/>
       <c r="D9" s="3"/>
       <c r="E9" s="3"/>
     </row>
-    <row r="10" spans="2:7" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:7" ht="26.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B10" s="3"/>
       <c r="C10" s="3"/>
       <c r="D10" s="3"/>
       <c r="E10" s="3"/>
     </row>
-    <row r="11" spans="2:7" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:7" ht="26.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B11" s="3"/>
       <c r="C11" s="3"/>
       <c r="D11" s="3"/>
       <c r="E11" s="3"/>
     </row>
-    <row r="12" spans="2:7" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:7" ht="26.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B12" s="3"/>
       <c r="C12" s="3"/>
       <c r="D12" s="3"/>
       <c r="E12" s="3"/>
     </row>
-    <row r="13" spans="2:7" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:7" ht="26.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B13" s="3"/>
       <c r="C13" s="3"/>
       <c r="D13" s="3"/>

</xml_diff>

<commit_message>
updated code and tables
pushed code update
</commit_message>
<xml_diff>
--- a/manuscript/BANTER_Pseudorca-AllTablesxlsx.xlsx
+++ b/manuscript/BANTER_Pseudorca-AllTablesxlsx.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yvonne.barkley\Github\BANTER_Pseudorca\manuscript\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66D9931E-3541-4DC1-BFF3-EEC28517D345}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8E8231D-35F1-4F35-9800-9E068DF56C4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="888" yWindow="768" windowWidth="31656" windowHeight="13224" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Threshold_Table" sheetId="4" r:id="rId1"/>
@@ -228,9 +228,6 @@
     <t>Suvery Year</t>
   </si>
   <si>
-    <t>(false +)</t>
-  </si>
-  <si>
     <t>Banter Threshold</t>
   </si>
   <si>
@@ -243,9 +240,6 @@
     <t xml:space="preserve">SSC </t>
   </si>
   <si>
-    <t>SA&amp;SSC</t>
-  </si>
-  <si>
     <t xml:space="preserve">Raw </t>
   </si>
   <si>
@@ -418,6 +412,12 @@
   </si>
   <si>
     <t>10; 11</t>
+  </si>
+  <si>
+    <t>(false positives)</t>
+  </si>
+  <si>
+    <t>SA &amp; SSC</t>
   </si>
 </sst>
 </file>
@@ -427,7 +427,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -464,8 +464,23 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
+      <sz val="16"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="16"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <i/>
-      <sz val="11"/>
+      <sz val="16"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -492,7 +507,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="21">
+  <borders count="23">
     <border>
       <left/>
       <right/>
@@ -754,11 +769,35 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -812,65 +851,71 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1152,389 +1197,385 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{16B82A36-BAB4-4DA2-945D-9C525C938092}">
-  <dimension ref="A1:Q8"/>
+  <dimension ref="B1:R14"/>
   <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="16.33203125" style="23" customWidth="1"/>
-    <col min="2" max="2" width="11.44140625" style="24" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="6.88671875" style="24" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="7.88671875" style="24" customWidth="1"/>
-    <col min="6" max="8" width="6.88671875" style="24" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="7.88671875" style="24" bestFit="1" customWidth="1"/>
-    <col min="10" max="12" width="5.88671875" style="24" bestFit="1" customWidth="1"/>
-    <col min="13" max="14" width="7.88671875" style="24" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="8.5546875" style="24" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="6.88671875" style="24" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="7.88671875" style="24" bestFit="1" customWidth="1"/>
-    <col min="18" max="16384" width="9.109375" style="24"/>
+    <col min="1" max="1" width="9.109375" style="24"/>
+    <col min="2" max="2" width="15.33203125" style="23" customWidth="1"/>
+    <col min="3" max="18" width="12.44140625" style="24" customWidth="1"/>
+    <col min="19" max="16384" width="9.109375" style="24"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="26"/>
-      <c r="B1" s="36" t="s">
+    <row r="1" spans="2:18" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="2" spans="2:18" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="B2" s="28"/>
+      <c r="C2" s="29" t="s">
         <v>61</v>
       </c>
-      <c r="C1" s="36"/>
-      <c r="D1" s="36"/>
-      <c r="E1" s="36"/>
-      <c r="F1" s="27"/>
-      <c r="G1" s="27"/>
-      <c r="H1" s="27"/>
-      <c r="I1" s="27"/>
-      <c r="J1" s="27"/>
-      <c r="K1" s="34"/>
-      <c r="L1" s="34"/>
-      <c r="M1" s="34"/>
-      <c r="N1" s="34"/>
-      <c r="O1" s="37" t="s">
+      <c r="D2" s="30"/>
+      <c r="E2" s="30"/>
+      <c r="F2" s="30"/>
+      <c r="G2" s="31"/>
+      <c r="H2" s="31"/>
+      <c r="I2" s="31"/>
+      <c r="J2" s="31"/>
+      <c r="K2" s="31"/>
+      <c r="L2" s="32"/>
+      <c r="M2" s="32"/>
+      <c r="N2" s="32"/>
+      <c r="O2" s="32"/>
+      <c r="P2" s="33"/>
+      <c r="Q2" s="32"/>
+      <c r="R2" s="34"/>
+    </row>
+    <row r="3" spans="2:18" ht="42" x14ac:dyDescent="0.4">
+      <c r="B3" s="46" t="s">
         <v>62</v>
       </c>
-      <c r="P1" s="34"/>
-      <c r="Q1" s="35"/>
-    </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A2" s="38" t="s">
+      <c r="C3" s="35">
+        <v>2017</v>
+      </c>
+      <c r="D3" s="31"/>
+      <c r="E3" s="31"/>
+      <c r="F3" s="36"/>
+      <c r="G3" s="35">
+        <v>2023</v>
+      </c>
+      <c r="H3" s="31"/>
+      <c r="I3" s="31"/>
+      <c r="J3" s="36"/>
+      <c r="K3" s="35">
+        <v>2024</v>
+      </c>
+      <c r="L3" s="32"/>
+      <c r="M3" s="32"/>
+      <c r="N3" s="34"/>
+      <c r="O3" s="35" t="s">
+        <v>50</v>
+      </c>
+      <c r="P3" s="32"/>
+      <c r="Q3" s="32"/>
+      <c r="R3" s="34"/>
+    </row>
+    <row r="4" spans="2:18" ht="21" x14ac:dyDescent="0.4">
+      <c r="B4" s="37"/>
+      <c r="C4" s="38" t="s">
         <v>63</v>
       </c>
-      <c r="B2" s="26">
-        <v>2017</v>
-      </c>
-      <c r="C2" s="27"/>
-      <c r="D2" s="27"/>
-      <c r="E2" s="28"/>
-      <c r="F2" s="26">
-        <v>2023</v>
-      </c>
-      <c r="G2" s="27"/>
-      <c r="H2" s="27"/>
-      <c r="I2" s="28"/>
-      <c r="J2" s="26">
-        <v>2024</v>
-      </c>
-      <c r="K2" s="34"/>
-      <c r="L2" s="34"/>
-      <c r="M2" s="35"/>
-      <c r="N2" s="26" t="s">
-        <v>50</v>
-      </c>
-      <c r="O2" s="34"/>
-      <c r="P2" s="34"/>
-      <c r="Q2" s="35"/>
-    </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A3" s="39"/>
-      <c r="B3" s="29" t="s">
+      <c r="D4" s="39" t="s">
         <v>64</v>
       </c>
-      <c r="C3" s="25" t="s">
+      <c r="E4" s="39" t="s">
         <v>65</v>
       </c>
-      <c r="D3" s="25" t="s">
+      <c r="F4" s="40" t="s">
+        <v>125</v>
+      </c>
+      <c r="G4" s="38" t="s">
         <v>66</v>
       </c>
-      <c r="E3" s="30" t="s">
+      <c r="H4" s="39" t="s">
+        <v>64</v>
+      </c>
+      <c r="I4" s="39" t="s">
+        <v>65</v>
+      </c>
+      <c r="J4" s="40" t="s">
+        <v>125</v>
+      </c>
+      <c r="K4" s="38" t="s">
+        <v>66</v>
+      </c>
+      <c r="L4" s="39" t="s">
+        <v>64</v>
+      </c>
+      <c r="M4" s="39" t="s">
+        <v>65</v>
+      </c>
+      <c r="N4" s="40" t="s">
+        <v>125</v>
+      </c>
+      <c r="O4" s="38" t="s">
+        <v>66</v>
+      </c>
+      <c r="P4" s="39" t="s">
+        <v>64</v>
+      </c>
+      <c r="Q4" s="39" t="s">
+        <v>65</v>
+      </c>
+      <c r="R4" s="40" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="5" spans="2:18" ht="21" x14ac:dyDescent="0.4">
+      <c r="B5" s="41">
+        <v>0.5</v>
+      </c>
+      <c r="C5" s="38" t="s">
         <v>67</v>
       </c>
-      <c r="F3" s="29" t="s">
+      <c r="D5" s="39" t="s">
         <v>68</v>
       </c>
-      <c r="G3" s="25" t="s">
-        <v>65</v>
-      </c>
-      <c r="H3" s="25" t="s">
-        <v>66</v>
-      </c>
-      <c r="I3" s="30" t="s">
-        <v>67</v>
-      </c>
-      <c r="J3" s="29" t="s">
-        <v>68</v>
-      </c>
-      <c r="K3" s="25" t="s">
-        <v>65</v>
-      </c>
-      <c r="L3" s="25" t="s">
-        <v>66</v>
-      </c>
-      <c r="M3" s="30" t="s">
-        <v>67</v>
-      </c>
-      <c r="N3" s="29" t="s">
-        <v>68</v>
-      </c>
-      <c r="O3" s="25" t="s">
-        <v>65</v>
-      </c>
-      <c r="P3" s="25" t="s">
-        <v>66</v>
-      </c>
-      <c r="Q3" s="30" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A4" s="40">
-        <v>0.5</v>
-      </c>
-      <c r="B4" s="29" t="s">
+      <c r="E5" s="39" t="s">
         <v>69</v>
       </c>
-      <c r="C4" s="25" t="s">
+      <c r="F5" s="40" t="s">
         <v>70</v>
       </c>
-      <c r="D4" s="25" t="s">
+      <c r="G5" s="38" t="s">
         <v>71</v>
       </c>
-      <c r="E4" s="30" t="s">
+      <c r="H5" s="39" t="s">
         <v>72</v>
       </c>
-      <c r="F4" s="29" t="s">
+      <c r="I5" s="39" t="s">
         <v>73</v>
       </c>
-      <c r="G4" s="25" t="s">
+      <c r="J5" s="40" t="s">
         <v>74</v>
       </c>
-      <c r="H4" s="25" t="s">
+      <c r="K5" s="38" t="s">
         <v>75</v>
       </c>
-      <c r="I4" s="30" t="s">
+      <c r="L5" s="39" t="s">
         <v>76</v>
       </c>
-      <c r="J4" s="29" t="s">
+      <c r="M5" s="39" t="s">
         <v>77</v>
       </c>
-      <c r="K4" s="25" t="s">
+      <c r="N5" s="40" t="s">
         <v>78</v>
       </c>
-      <c r="L4" s="25" t="s">
+      <c r="O5" s="38" t="s">
         <v>79</v>
       </c>
-      <c r="M4" s="30" t="s">
+      <c r="P5" s="39" t="s">
         <v>80</v>
       </c>
-      <c r="N4" s="29" t="s">
+      <c r="Q5" s="39" t="s">
         <v>81</v>
       </c>
-      <c r="O4" s="25" t="s">
+      <c r="R5" s="40" t="s">
         <v>82</v>
       </c>
-      <c r="P4" s="25" t="s">
+    </row>
+    <row r="6" spans="2:18" ht="21" x14ac:dyDescent="0.4">
+      <c r="B6" s="41">
+        <v>0.6</v>
+      </c>
+      <c r="C6" s="38" t="s">
         <v>83</v>
       </c>
-      <c r="Q4" s="30" t="s">
+      <c r="D6" s="39" t="s">
         <v>84</v>
       </c>
-    </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A5" s="40">
-        <v>0.6</v>
-      </c>
-      <c r="B5" s="29" t="s">
+      <c r="E6" s="39" t="s">
         <v>85</v>
       </c>
-      <c r="C5" s="25" t="s">
+      <c r="F6" s="40" t="s">
+        <v>70</v>
+      </c>
+      <c r="G6" s="38" t="s">
         <v>86</v>
       </c>
-      <c r="D5" s="25" t="s">
+      <c r="H6" s="39" t="s">
         <v>87</v>
       </c>
-      <c r="E5" s="30" t="s">
-        <v>72</v>
-      </c>
-      <c r="F5" s="29" t="s">
+      <c r="I6" s="39" t="s">
         <v>88</v>
       </c>
-      <c r="G5" s="25" t="s">
+      <c r="J6" s="40" t="s">
+        <v>78</v>
+      </c>
+      <c r="K6" s="38" t="s">
         <v>89</v>
       </c>
-      <c r="H5" s="25" t="s">
+      <c r="L6" s="39" t="s">
         <v>90</v>
       </c>
-      <c r="I5" s="30" t="s">
-        <v>80</v>
-      </c>
-      <c r="J5" s="29" t="s">
+      <c r="M6" s="39" t="s">
+        <v>89</v>
+      </c>
+      <c r="N6" s="40" t="s">
+        <v>90</v>
+      </c>
+      <c r="O6" s="38" t="s">
+        <v>81</v>
+      </c>
+      <c r="P6" s="39" t="s">
         <v>91</v>
       </c>
-      <c r="K5" s="25" t="s">
+      <c r="Q6" s="39" t="s">
         <v>92</v>
       </c>
-      <c r="L5" s="25" t="s">
-        <v>91</v>
-      </c>
-      <c r="M5" s="30" t="s">
-        <v>92</v>
-      </c>
-      <c r="N5" s="29" t="s">
-        <v>83</v>
-      </c>
-      <c r="O5" s="25" t="s">
+      <c r="R6" s="40" t="s">
         <v>93</v>
       </c>
-      <c r="P5" s="25" t="s">
+    </row>
+    <row r="7" spans="2:18" ht="21" x14ac:dyDescent="0.4">
+      <c r="B7" s="41">
+        <v>0.7</v>
+      </c>
+      <c r="C7" s="38" t="s">
         <v>94</v>
       </c>
-      <c r="Q5" s="30" t="s">
+      <c r="D7" s="39" t="s">
         <v>95</v>
       </c>
-    </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A6" s="40">
-        <v>0.7</v>
-      </c>
-      <c r="B6" s="29" t="s">
+      <c r="E7" s="39" t="s">
         <v>96</v>
       </c>
-      <c r="C6" s="25" t="s">
+      <c r="F7" s="40" t="s">
         <v>97</v>
       </c>
-      <c r="D6" s="25" t="s">
+      <c r="G7" s="38" t="s">
         <v>98</v>
       </c>
-      <c r="E6" s="30" t="s">
+      <c r="H7" s="39" t="s">
         <v>99</v>
       </c>
-      <c r="F6" s="29" t="s">
+      <c r="I7" s="39" t="s">
         <v>100</v>
       </c>
-      <c r="G6" s="25" t="s">
+      <c r="J7" s="40" t="s">
         <v>101</v>
       </c>
-      <c r="H6" s="25" t="s">
+      <c r="K7" s="38" t="s">
         <v>102</v>
       </c>
-      <c r="I6" s="30" t="s">
+      <c r="L7" s="39" t="s">
+        <v>101</v>
+      </c>
+      <c r="M7" s="39" t="s">
+        <v>102</v>
+      </c>
+      <c r="N7" s="40" t="s">
+        <v>101</v>
+      </c>
+      <c r="O7" s="38" t="s">
         <v>103</v>
       </c>
-      <c r="J6" s="29" t="s">
+      <c r="P7" s="39" t="s">
         <v>104</v>
       </c>
-      <c r="K6" s="25" t="s">
-        <v>103</v>
-      </c>
-      <c r="L6" s="25" t="s">
-        <v>104</v>
-      </c>
-      <c r="M6" s="30" t="s">
-        <v>103</v>
-      </c>
-      <c r="N6" s="29" t="s">
+      <c r="Q7" s="39" t="s">
         <v>105</v>
       </c>
-      <c r="O6" s="25" t="s">
+      <c r="R7" s="40" t="s">
         <v>106</v>
       </c>
-      <c r="P6" s="25" t="s">
+    </row>
+    <row r="8" spans="2:18" ht="21" x14ac:dyDescent="0.4">
+      <c r="B8" s="41">
+        <v>0.8</v>
+      </c>
+      <c r="C8" s="38" t="s">
         <v>107</v>
       </c>
-      <c r="Q6" s="30" t="s">
+      <c r="D8" s="39" t="s">
         <v>108</v>
       </c>
-    </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A7" s="40">
-        <v>0.8</v>
-      </c>
-      <c r="B7" s="29" t="s">
+      <c r="E8" s="39" t="s">
+        <v>107</v>
+      </c>
+      <c r="F8" s="40" t="s">
+        <v>108</v>
+      </c>
+      <c r="G8" s="38" t="s">
         <v>109</v>
       </c>
-      <c r="C7" s="25" t="s">
+      <c r="H8" s="39" t="s">
         <v>110</v>
       </c>
-      <c r="D7" s="25" t="s">
-        <v>109</v>
-      </c>
-      <c r="E7" s="30" t="s">
+      <c r="I8" s="39" t="s">
         <v>110</v>
       </c>
-      <c r="F7" s="29" t="s">
+      <c r="J8" s="40" t="s">
         <v>111</v>
       </c>
-      <c r="G7" s="25" t="s">
+      <c r="K8" s="38" t="s">
         <v>112</v>
       </c>
-      <c r="H7" s="25" t="s">
+      <c r="L8" s="39" t="s">
         <v>112</v>
       </c>
-      <c r="I7" s="30" t="s">
+      <c r="M8" s="39" t="s">
+        <v>112</v>
+      </c>
+      <c r="N8" s="40" t="s">
+        <v>112</v>
+      </c>
+      <c r="O8" s="38" t="s">
         <v>113</v>
       </c>
-      <c r="J7" s="29" t="s">
+      <c r="P8" s="39" t="s">
         <v>114</v>
       </c>
-      <c r="K7" s="25" t="s">
-        <v>114</v>
-      </c>
-      <c r="L7" s="25" t="s">
-        <v>114</v>
-      </c>
-      <c r="M7" s="30" t="s">
-        <v>114</v>
-      </c>
-      <c r="N7" s="29" t="s">
+      <c r="Q8" s="39" t="s">
         <v>115</v>
       </c>
-      <c r="O7" s="25" t="s">
+      <c r="R8" s="40" t="s">
         <v>116</v>
       </c>
-      <c r="P7" s="25" t="s">
+    </row>
+    <row r="9" spans="2:18" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="B9" s="42">
+        <v>0.9</v>
+      </c>
+      <c r="C9" s="43" t="s">
+        <v>112</v>
+      </c>
+      <c r="D9" s="44" t="s">
+        <v>112</v>
+      </c>
+      <c r="E9" s="44" t="s">
+        <v>112</v>
+      </c>
+      <c r="F9" s="45" t="s">
+        <v>112</v>
+      </c>
+      <c r="G9" s="43" t="s">
         <v>117</v>
       </c>
-      <c r="Q7" s="30" t="s">
+      <c r="H9" s="44" t="s">
+        <v>117</v>
+      </c>
+      <c r="I9" s="44" t="s">
+        <v>117</v>
+      </c>
+      <c r="J9" s="45" t="s">
+        <v>117</v>
+      </c>
+      <c r="K9" s="43" t="s">
+        <v>117</v>
+      </c>
+      <c r="L9" s="44" t="s">
+        <v>117</v>
+      </c>
+      <c r="M9" s="44" t="s">
+        <v>117</v>
+      </c>
+      <c r="N9" s="45" t="s">
+        <v>117</v>
+      </c>
+      <c r="O9" s="43" t="s">
         <v>118</v>
       </c>
-    </row>
-    <row r="8" spans="1:17" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="41">
-        <v>0.9</v>
-      </c>
-      <c r="B8" s="31" t="s">
-        <v>114</v>
-      </c>
-      <c r="C8" s="32" t="s">
-        <v>114</v>
-      </c>
-      <c r="D8" s="32" t="s">
-        <v>114</v>
-      </c>
-      <c r="E8" s="33" t="s">
-        <v>114</v>
-      </c>
-      <c r="F8" s="31" t="s">
-        <v>119</v>
-      </c>
-      <c r="G8" s="32" t="s">
-        <v>119</v>
-      </c>
-      <c r="H8" s="32" t="s">
-        <v>119</v>
-      </c>
-      <c r="I8" s="33" t="s">
-        <v>119</v>
-      </c>
-      <c r="J8" s="31" t="s">
-        <v>119</v>
-      </c>
-      <c r="K8" s="32" t="s">
-        <v>119</v>
-      </c>
-      <c r="L8" s="32" t="s">
-        <v>119</v>
-      </c>
-      <c r="M8" s="33" t="s">
-        <v>119</v>
-      </c>
-      <c r="N8" s="31" t="s">
-        <v>120</v>
-      </c>
-      <c r="O8" s="32" t="s">
-        <v>120</v>
-      </c>
-      <c r="P8" s="32" t="s">
-        <v>120</v>
-      </c>
-      <c r="Q8" s="33" t="s">
-        <v>120</v>
+      <c r="P9" s="44" t="s">
+        <v>118</v>
+      </c>
+      <c r="Q9" s="44" t="s">
+        <v>118</v>
+      </c>
+      <c r="R9" s="45" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="14" spans="2:18" x14ac:dyDescent="0.3">
+      <c r="C14" s="24" t="s">
+        <v>124</v>
       </c>
     </row>
   </sheetData>
@@ -1565,7 +1606,7 @@
       <c r="E2" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="F2" s="43" t="s">
+      <c r="F2" s="25" t="s">
         <v>3</v>
       </c>
       <c r="G2" s="12" t="s">
@@ -1581,10 +1622,10 @@
         <v>18</v>
       </c>
       <c r="K2" s="12" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="L2" s="12" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="M2" s="12" t="s">
         <v>4</v>
@@ -1616,8 +1657,8 @@
       <c r="J3" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="K3" s="44" t="s">
-        <v>123</v>
+      <c r="K3" s="26" t="s">
+        <v>121</v>
       </c>
       <c r="L3" s="2"/>
       <c r="M3" s="14"/>
@@ -1646,7 +1687,7 @@
       <c r="J4" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="K4" s="44">
+      <c r="K4" s="26">
         <v>2</v>
       </c>
       <c r="L4" s="2"/>
@@ -1678,7 +1719,7 @@
       <c r="J5" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="K5" s="44">
+      <c r="K5" s="26">
         <v>1</v>
       </c>
       <c r="L5" s="2"/>
@@ -1786,7 +1827,7 @@
         <v>5</v>
       </c>
       <c r="D9" s="13" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="E9" s="14" t="s">
         <v>13</v>
@@ -1805,7 +1846,7 @@
         <v>19</v>
       </c>
       <c r="K9" s="2" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="L9" s="2"/>
       <c r="M9" s="14"/>
@@ -2322,9 +2363,9 @@
   </cols>
   <sheetData>
     <row r="3" spans="2:7" ht="26.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="C3" s="42"/>
-      <c r="D3" s="42"/>
-      <c r="E3" s="42"/>
+      <c r="C3" s="27"/>
+      <c r="D3" s="27"/>
+      <c r="E3" s="27"/>
     </row>
     <row r="4" spans="2:7" ht="56.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B4" s="4"/>

</xml_diff>

<commit_message>
code updates, Supp table update
Precision recall updates, added more info to Table S1
</commit_message>
<xml_diff>
--- a/manuscript/BANTER_Pseudorca-AllTablesxlsx.xlsx
+++ b/manuscript/BANTER_Pseudorca-AllTablesxlsx.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yvonne.barkley\Github\BANTER_Pseudorca\manuscript\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8E8231D-35F1-4F35-9800-9E068DF56C4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37A33E58-30D1-43E4-8D29-ABDD14ED5008}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="888" yWindow="768" windowWidth="31656" windowHeight="13224" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38280" yWindow="4140" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Threshold_Table" sheetId="4" r:id="rId1"/>
@@ -39,8 +39,42 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>Reviewer</author>
+  </authors>
+  <commentList>
+    <comment ref="O2" authorId="0" shapeId="0" xr:uid="{F3D028D6-C6F0-40AC-98AD-084147D6A7A6}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Reviewer:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+YB - Not including since it's so variable and hard to understand.</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="205" uniqueCount="126">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="218" uniqueCount="128">
   <si>
     <t>Survey Year</t>
   </si>
@@ -54,9 +88,6 @@
     <t>Minimum &amp; Maximum Hydrophone Spacing</t>
   </si>
   <si>
-    <t>References for more details</t>
-  </si>
-  <si>
     <t>Hawaiian EEZ</t>
   </si>
   <si>
@@ -90,9 +121,6 @@
     <t>Hydrophone Flat Frequency Response</t>
   </si>
   <si>
-    <t>2-40 kHz</t>
-  </si>
-  <si>
     <t>2.02.7b</t>
   </si>
   <si>
@@ -117,12 +145,6 @@
     <t>Visually Verified Pc</t>
   </si>
   <si>
-    <t>Sampling Rate (kHz)</t>
-  </si>
-  <si>
-    <t>2–85 kHz</t>
-  </si>
-  <si>
     <t>Total Acoustic Hours</t>
   </si>
   <si>
@@ -418,6 +440,24 @@
   </si>
   <si>
     <t>SA &amp; SSC</t>
+  </si>
+  <si>
+    <t>References for more details about the survey</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sampling Rate </t>
+  </si>
+  <si>
+    <t>192 kHz</t>
+  </si>
+  <si>
+    <t>500 kHz</t>
+  </si>
+  <si>
+    <t>2 - 40 kHz</t>
+  </si>
+  <si>
+    <t>2 – 85 kHz</t>
   </si>
 </sst>
 </file>
@@ -427,7 +467,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -486,6 +526,25 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -797,7 +856,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -854,68 +913,71 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1208,374 +1270,374 @@
   <sheetData>
     <row r="1" spans="2:18" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="2" spans="2:18" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="B2" s="28"/>
-      <c r="C2" s="29" t="s">
+      <c r="B2" s="26"/>
+      <c r="C2" s="27" t="s">
+        <v>57</v>
+      </c>
+      <c r="D2" s="28"/>
+      <c r="E2" s="28"/>
+      <c r="F2" s="28"/>
+      <c r="G2" s="29"/>
+      <c r="H2" s="29"/>
+      <c r="I2" s="29"/>
+      <c r="J2" s="29"/>
+      <c r="K2" s="29"/>
+      <c r="L2" s="30"/>
+      <c r="M2" s="30"/>
+      <c r="N2" s="30"/>
+      <c r="O2" s="30"/>
+      <c r="P2" s="31"/>
+      <c r="Q2" s="30"/>
+      <c r="R2" s="32"/>
+    </row>
+    <row r="3" spans="2:18" ht="42" x14ac:dyDescent="0.4">
+      <c r="B3" s="44" t="s">
+        <v>58</v>
+      </c>
+      <c r="C3" s="33">
+        <v>2017</v>
+      </c>
+      <c r="D3" s="29"/>
+      <c r="E3" s="29"/>
+      <c r="F3" s="34"/>
+      <c r="G3" s="33">
+        <v>2023</v>
+      </c>
+      <c r="H3" s="29"/>
+      <c r="I3" s="29"/>
+      <c r="J3" s="34"/>
+      <c r="K3" s="33">
+        <v>2024</v>
+      </c>
+      <c r="L3" s="30"/>
+      <c r="M3" s="30"/>
+      <c r="N3" s="32"/>
+      <c r="O3" s="33" t="s">
+        <v>46</v>
+      </c>
+      <c r="P3" s="30"/>
+      <c r="Q3" s="30"/>
+      <c r="R3" s="32"/>
+    </row>
+    <row r="4" spans="2:18" ht="21" x14ac:dyDescent="0.4">
+      <c r="B4" s="35"/>
+      <c r="C4" s="36" t="s">
+        <v>59</v>
+      </c>
+      <c r="D4" s="37" t="s">
+        <v>60</v>
+      </c>
+      <c r="E4" s="37" t="s">
         <v>61</v>
       </c>
-      <c r="D2" s="30"/>
-      <c r="E2" s="30"/>
-      <c r="F2" s="30"/>
-      <c r="G2" s="31"/>
-      <c r="H2" s="31"/>
-      <c r="I2" s="31"/>
-      <c r="J2" s="31"/>
-      <c r="K2" s="31"/>
-      <c r="L2" s="32"/>
-      <c r="M2" s="32"/>
-      <c r="N2" s="32"/>
-      <c r="O2" s="32"/>
-      <c r="P2" s="33"/>
-      <c r="Q2" s="32"/>
-      <c r="R2" s="34"/>
-    </row>
-    <row r="3" spans="2:18" ht="42" x14ac:dyDescent="0.4">
-      <c r="B3" s="46" t="s">
+      <c r="F4" s="38" t="s">
+        <v>121</v>
+      </c>
+      <c r="G4" s="36" t="s">
         <v>62</v>
       </c>
-      <c r="C3" s="35">
-        <v>2017</v>
-      </c>
-      <c r="D3" s="31"/>
-      <c r="E3" s="31"/>
-      <c r="F3" s="36"/>
-      <c r="G3" s="35">
-        <v>2023</v>
-      </c>
-      <c r="H3" s="31"/>
-      <c r="I3" s="31"/>
-      <c r="J3" s="36"/>
-      <c r="K3" s="35">
-        <v>2024</v>
-      </c>
-      <c r="L3" s="32"/>
-      <c r="M3" s="32"/>
-      <c r="N3" s="34"/>
-      <c r="O3" s="35" t="s">
-        <v>50</v>
-      </c>
-      <c r="P3" s="32"/>
-      <c r="Q3" s="32"/>
-      <c r="R3" s="34"/>
-    </row>
-    <row r="4" spans="2:18" ht="21" x14ac:dyDescent="0.4">
-      <c r="B4" s="37"/>
-      <c r="C4" s="38" t="s">
+      <c r="H4" s="37" t="s">
+        <v>60</v>
+      </c>
+      <c r="I4" s="37" t="s">
+        <v>61</v>
+      </c>
+      <c r="J4" s="38" t="s">
+        <v>121</v>
+      </c>
+      <c r="K4" s="36" t="s">
+        <v>62</v>
+      </c>
+      <c r="L4" s="37" t="s">
+        <v>60</v>
+      </c>
+      <c r="M4" s="37" t="s">
+        <v>61</v>
+      </c>
+      <c r="N4" s="38" t="s">
+        <v>121</v>
+      </c>
+      <c r="O4" s="36" t="s">
+        <v>62</v>
+      </c>
+      <c r="P4" s="37" t="s">
+        <v>60</v>
+      </c>
+      <c r="Q4" s="37" t="s">
+        <v>61</v>
+      </c>
+      <c r="R4" s="38" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="5" spans="2:18" ht="21" x14ac:dyDescent="0.4">
+      <c r="B5" s="39">
+        <v>0.5</v>
+      </c>
+      <c r="C5" s="36" t="s">
         <v>63</v>
       </c>
-      <c r="D4" s="39" t="s">
+      <c r="D5" s="37" t="s">
         <v>64</v>
       </c>
-      <c r="E4" s="39" t="s">
+      <c r="E5" s="37" t="s">
         <v>65</v>
       </c>
-      <c r="F4" s="40" t="s">
-        <v>125</v>
-      </c>
-      <c r="G4" s="38" t="s">
+      <c r="F5" s="38" t="s">
         <v>66</v>
       </c>
-      <c r="H4" s="39" t="s">
-        <v>64</v>
-      </c>
-      <c r="I4" s="39" t="s">
-        <v>65</v>
-      </c>
-      <c r="J4" s="40" t="s">
-        <v>125</v>
-      </c>
-      <c r="K4" s="38" t="s">
+      <c r="G5" s="36" t="s">
+        <v>67</v>
+      </c>
+      <c r="H5" s="37" t="s">
+        <v>68</v>
+      </c>
+      <c r="I5" s="37" t="s">
+        <v>69</v>
+      </c>
+      <c r="J5" s="38" t="s">
+        <v>70</v>
+      </c>
+      <c r="K5" s="36" t="s">
+        <v>71</v>
+      </c>
+      <c r="L5" s="37" t="s">
+        <v>72</v>
+      </c>
+      <c r="M5" s="37" t="s">
+        <v>73</v>
+      </c>
+      <c r="N5" s="38" t="s">
+        <v>74</v>
+      </c>
+      <c r="O5" s="36" t="s">
+        <v>75</v>
+      </c>
+      <c r="P5" s="37" t="s">
+        <v>76</v>
+      </c>
+      <c r="Q5" s="37" t="s">
+        <v>77</v>
+      </c>
+      <c r="R5" s="38" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="6" spans="2:18" ht="21" x14ac:dyDescent="0.4">
+      <c r="B6" s="39">
+        <v>0.6</v>
+      </c>
+      <c r="C6" s="36" t="s">
+        <v>79</v>
+      </c>
+      <c r="D6" s="37" t="s">
+        <v>80</v>
+      </c>
+      <c r="E6" s="37" t="s">
+        <v>81</v>
+      </c>
+      <c r="F6" s="38" t="s">
         <v>66</v>
       </c>
-      <c r="L4" s="39" t="s">
-        <v>64</v>
-      </c>
-      <c r="M4" s="39" t="s">
-        <v>65</v>
-      </c>
-      <c r="N4" s="40" t="s">
-        <v>125</v>
-      </c>
-      <c r="O4" s="38" t="s">
-        <v>66</v>
-      </c>
-      <c r="P4" s="39" t="s">
-        <v>64</v>
-      </c>
-      <c r="Q4" s="39" t="s">
-        <v>65</v>
-      </c>
-      <c r="R4" s="40" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="5" spans="2:18" ht="21" x14ac:dyDescent="0.4">
-      <c r="B5" s="41">
-        <v>0.5</v>
-      </c>
-      <c r="C5" s="38" t="s">
-        <v>67</v>
-      </c>
-      <c r="D5" s="39" t="s">
-        <v>68</v>
-      </c>
-      <c r="E5" s="39" t="s">
-        <v>69</v>
-      </c>
-      <c r="F5" s="40" t="s">
-        <v>70</v>
-      </c>
-      <c r="G5" s="38" t="s">
-        <v>71</v>
-      </c>
-      <c r="H5" s="39" t="s">
-        <v>72</v>
-      </c>
-      <c r="I5" s="39" t="s">
-        <v>73</v>
-      </c>
-      <c r="J5" s="40" t="s">
+      <c r="G6" s="36" t="s">
+        <v>82</v>
+      </c>
+      <c r="H6" s="37" t="s">
+        <v>83</v>
+      </c>
+      <c r="I6" s="37" t="s">
+        <v>84</v>
+      </c>
+      <c r="J6" s="38" t="s">
         <v>74</v>
       </c>
-      <c r="K5" s="38" t="s">
-        <v>75</v>
-      </c>
-      <c r="L5" s="39" t="s">
-        <v>76</v>
-      </c>
-      <c r="M5" s="39" t="s">
+      <c r="K6" s="36" t="s">
+        <v>85</v>
+      </c>
+      <c r="L6" s="37" t="s">
+        <v>86</v>
+      </c>
+      <c r="M6" s="37" t="s">
+        <v>85</v>
+      </c>
+      <c r="N6" s="38" t="s">
+        <v>86</v>
+      </c>
+      <c r="O6" s="36" t="s">
         <v>77</v>
       </c>
-      <c r="N5" s="40" t="s">
-        <v>78</v>
-      </c>
-      <c r="O5" s="38" t="s">
-        <v>79</v>
-      </c>
-      <c r="P5" s="39" t="s">
-        <v>80</v>
-      </c>
-      <c r="Q5" s="39" t="s">
-        <v>81</v>
-      </c>
-      <c r="R5" s="40" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="6" spans="2:18" ht="21" x14ac:dyDescent="0.4">
-      <c r="B6" s="41">
-        <v>0.6</v>
-      </c>
-      <c r="C6" s="38" t="s">
-        <v>83</v>
-      </c>
-      <c r="D6" s="39" t="s">
-        <v>84</v>
-      </c>
-      <c r="E6" s="39" t="s">
-        <v>85</v>
-      </c>
-      <c r="F6" s="40" t="s">
-        <v>70</v>
-      </c>
-      <c r="G6" s="38" t="s">
-        <v>86</v>
-      </c>
-      <c r="H6" s="39" t="s">
+      <c r="P6" s="37" t="s">
         <v>87</v>
       </c>
-      <c r="I6" s="39" t="s">
+      <c r="Q6" s="37" t="s">
         <v>88</v>
       </c>
-      <c r="J6" s="40" t="s">
-        <v>78</v>
-      </c>
-      <c r="K6" s="38" t="s">
+      <c r="R6" s="38" t="s">
         <v>89</v>
       </c>
-      <c r="L6" s="39" t="s">
+    </row>
+    <row r="7" spans="2:18" ht="21" x14ac:dyDescent="0.4">
+      <c r="B7" s="39">
+        <v>0.7</v>
+      </c>
+      <c r="C7" s="36" t="s">
         <v>90</v>
       </c>
-      <c r="M6" s="39" t="s">
-        <v>89</v>
-      </c>
-      <c r="N6" s="40" t="s">
-        <v>90</v>
-      </c>
-      <c r="O6" s="38" t="s">
-        <v>81</v>
-      </c>
-      <c r="P6" s="39" t="s">
+      <c r="D7" s="37" t="s">
         <v>91</v>
       </c>
-      <c r="Q6" s="39" t="s">
+      <c r="E7" s="37" t="s">
         <v>92</v>
       </c>
-      <c r="R6" s="40" t="s">
+      <c r="F7" s="38" t="s">
         <v>93</v>
       </c>
-    </row>
-    <row r="7" spans="2:18" ht="21" x14ac:dyDescent="0.4">
-      <c r="B7" s="41">
-        <v>0.7</v>
-      </c>
-      <c r="C7" s="38" t="s">
+      <c r="G7" s="36" t="s">
         <v>94</v>
       </c>
-      <c r="D7" s="39" t="s">
+      <c r="H7" s="37" t="s">
         <v>95</v>
       </c>
-      <c r="E7" s="39" t="s">
+      <c r="I7" s="37" t="s">
         <v>96</v>
       </c>
-      <c r="F7" s="40" t="s">
+      <c r="J7" s="38" t="s">
         <v>97</v>
       </c>
-      <c r="G7" s="38" t="s">
+      <c r="K7" s="36" t="s">
         <v>98</v>
       </c>
-      <c r="H7" s="39" t="s">
+      <c r="L7" s="37" t="s">
+        <v>97</v>
+      </c>
+      <c r="M7" s="37" t="s">
+        <v>98</v>
+      </c>
+      <c r="N7" s="38" t="s">
+        <v>97</v>
+      </c>
+      <c r="O7" s="36" t="s">
         <v>99</v>
       </c>
-      <c r="I7" s="39" t="s">
+      <c r="P7" s="37" t="s">
         <v>100</v>
       </c>
-      <c r="J7" s="40" t="s">
+      <c r="Q7" s="37" t="s">
         <v>101</v>
       </c>
-      <c r="K7" s="38" t="s">
+      <c r="R7" s="38" t="s">
         <v>102</v>
       </c>
-      <c r="L7" s="39" t="s">
-        <v>101</v>
-      </c>
-      <c r="M7" s="39" t="s">
-        <v>102</v>
-      </c>
-      <c r="N7" s="40" t="s">
-        <v>101</v>
-      </c>
-      <c r="O7" s="38" t="s">
+    </row>
+    <row r="8" spans="2:18" ht="21" x14ac:dyDescent="0.4">
+      <c r="B8" s="39">
+        <v>0.8</v>
+      </c>
+      <c r="C8" s="36" t="s">
         <v>103</v>
       </c>
-      <c r="P7" s="39" t="s">
+      <c r="D8" s="37" t="s">
         <v>104</v>
       </c>
-      <c r="Q7" s="39" t="s">
+      <c r="E8" s="37" t="s">
+        <v>103</v>
+      </c>
+      <c r="F8" s="38" t="s">
+        <v>104</v>
+      </c>
+      <c r="G8" s="36" t="s">
         <v>105</v>
       </c>
-      <c r="R7" s="40" t="s">
+      <c r="H8" s="37" t="s">
         <v>106</v>
       </c>
-    </row>
-    <row r="8" spans="2:18" ht="21" x14ac:dyDescent="0.4">
-      <c r="B8" s="41">
-        <v>0.8</v>
-      </c>
-      <c r="C8" s="38" t="s">
+      <c r="I8" s="37" t="s">
+        <v>106</v>
+      </c>
+      <c r="J8" s="38" t="s">
         <v>107</v>
       </c>
-      <c r="D8" s="39" t="s">
+      <c r="K8" s="36" t="s">
         <v>108</v>
       </c>
-      <c r="E8" s="39" t="s">
-        <v>107</v>
-      </c>
-      <c r="F8" s="40" t="s">
+      <c r="L8" s="37" t="s">
         <v>108</v>
       </c>
-      <c r="G8" s="38" t="s">
+      <c r="M8" s="37" t="s">
+        <v>108</v>
+      </c>
+      <c r="N8" s="38" t="s">
+        <v>108</v>
+      </c>
+      <c r="O8" s="36" t="s">
         <v>109</v>
       </c>
-      <c r="H8" s="39" t="s">
+      <c r="P8" s="37" t="s">
         <v>110</v>
       </c>
-      <c r="I8" s="39" t="s">
-        <v>110</v>
-      </c>
-      <c r="J8" s="40" t="s">
+      <c r="Q8" s="37" t="s">
         <v>111</v>
       </c>
-      <c r="K8" s="38" t="s">
+      <c r="R8" s="38" t="s">
         <v>112</v>
       </c>
-      <c r="L8" s="39" t="s">
-        <v>112</v>
-      </c>
-      <c r="M8" s="39" t="s">
-        <v>112</v>
-      </c>
-      <c r="N8" s="40" t="s">
-        <v>112</v>
-      </c>
-      <c r="O8" s="38" t="s">
+    </row>
+    <row r="9" spans="2:18" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="B9" s="40">
+        <v>0.9</v>
+      </c>
+      <c r="C9" s="41" t="s">
+        <v>108</v>
+      </c>
+      <c r="D9" s="42" t="s">
+        <v>108</v>
+      </c>
+      <c r="E9" s="42" t="s">
+        <v>108</v>
+      </c>
+      <c r="F9" s="43" t="s">
+        <v>108</v>
+      </c>
+      <c r="G9" s="41" t="s">
         <v>113</v>
       </c>
-      <c r="P8" s="39" t="s">
+      <c r="H9" s="42" t="s">
+        <v>113</v>
+      </c>
+      <c r="I9" s="42" t="s">
+        <v>113</v>
+      </c>
+      <c r="J9" s="43" t="s">
+        <v>113</v>
+      </c>
+      <c r="K9" s="41" t="s">
+        <v>113</v>
+      </c>
+      <c r="L9" s="42" t="s">
+        <v>113</v>
+      </c>
+      <c r="M9" s="42" t="s">
+        <v>113</v>
+      </c>
+      <c r="N9" s="43" t="s">
+        <v>113</v>
+      </c>
+      <c r="O9" s="41" t="s">
         <v>114</v>
       </c>
-      <c r="Q8" s="39" t="s">
-        <v>115</v>
-      </c>
-      <c r="R8" s="40" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="9" spans="2:18" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="B9" s="42">
-        <v>0.9</v>
-      </c>
-      <c r="C9" s="43" t="s">
-        <v>112</v>
-      </c>
-      <c r="D9" s="44" t="s">
-        <v>112</v>
-      </c>
-      <c r="E9" s="44" t="s">
-        <v>112</v>
-      </c>
-      <c r="F9" s="45" t="s">
-        <v>112</v>
-      </c>
-      <c r="G9" s="43" t="s">
-        <v>117</v>
-      </c>
-      <c r="H9" s="44" t="s">
-        <v>117</v>
-      </c>
-      <c r="I9" s="44" t="s">
-        <v>117</v>
-      </c>
-      <c r="J9" s="45" t="s">
-        <v>117</v>
-      </c>
-      <c r="K9" s="43" t="s">
-        <v>117</v>
-      </c>
-      <c r="L9" s="44" t="s">
-        <v>117</v>
-      </c>
-      <c r="M9" s="44" t="s">
-        <v>117</v>
-      </c>
-      <c r="N9" s="45" t="s">
-        <v>117</v>
-      </c>
-      <c r="O9" s="43" t="s">
-        <v>118</v>
-      </c>
-      <c r="P9" s="44" t="s">
-        <v>118</v>
-      </c>
-      <c r="Q9" s="44" t="s">
-        <v>118</v>
-      </c>
-      <c r="R9" s="45" t="s">
-        <v>118</v>
+      <c r="P9" s="42" t="s">
+        <v>114</v>
+      </c>
+      <c r="Q9" s="42" t="s">
+        <v>114</v>
+      </c>
+      <c r="R9" s="43" t="s">
+        <v>114</v>
       </c>
     </row>
     <row r="14" spans="2:18" x14ac:dyDescent="0.3">
       <c r="C14" s="24" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
     </row>
   </sheetData>
@@ -1585,15 +1647,17 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B2:M15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="B2:O15"/>
   <sheetFormatPr defaultColWidth="14.33203125" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="10" customWidth="1"/>
-    <col min="3" max="4" width="23.33203125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="23.33203125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="17.21875" style="1" customWidth="1"/>
+    <col min="12" max="12" width="23.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:13" ht="83.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:15" ht="83.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B2" s="12" t="s">
         <v>0</v>
       </c>
@@ -1601,431 +1665,435 @@
         <v>1</v>
       </c>
       <c r="D2" s="12" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="E2" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="F2" s="25" t="s">
+      <c r="F2" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="G2" s="12" t="s">
+        <v>123</v>
+      </c>
+      <c r="H2" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="I2" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="J2" s="12" t="s">
+        <v>115</v>
+      </c>
+      <c r="K2" s="12" t="s">
+        <v>116</v>
+      </c>
+      <c r="L2" s="12" t="s">
+        <v>122</v>
+      </c>
+      <c r="O2" s="25" t="s">
         <v>3</v>
       </c>
-      <c r="G2" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="H2" s="12" t="s">
-        <v>25</v>
-      </c>
-      <c r="I2" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="J2" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="K2" s="12" t="s">
-        <v>119</v>
-      </c>
-      <c r="L2" s="12" t="s">
-        <v>120</v>
-      </c>
-      <c r="M2" s="12" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="3" spans="2:13" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="3" spans="2:15" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B3" s="12">
         <v>2010</v>
       </c>
       <c r="C3" s="13" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D3" s="13" t="s">
-        <v>47</v>
-      </c>
-      <c r="E3" s="14" t="s">
-        <v>11</v>
-      </c>
-      <c r="F3" s="14"/>
-      <c r="G3" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="H3" s="14">
-        <v>192</v>
-      </c>
-      <c r="I3" s="14">
+        <v>43</v>
+      </c>
+      <c r="E3" s="46" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3" s="46" t="s">
+        <v>126</v>
+      </c>
+      <c r="G3" s="46" t="s">
+        <v>124</v>
+      </c>
+      <c r="H3" s="46">
         <v>1445</v>
       </c>
-      <c r="J3" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="K3" s="26" t="s">
-        <v>121</v>
-      </c>
-      <c r="L3" s="2"/>
-      <c r="M3" s="14"/>
-    </row>
-    <row r="4" spans="2:13" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="I3" s="47" t="s">
+        <v>15</v>
+      </c>
+      <c r="J3" s="47" t="s">
+        <v>117</v>
+      </c>
+      <c r="K3" s="2"/>
+      <c r="L3" s="14"/>
+      <c r="O3" s="46"/>
+    </row>
+    <row r="4" spans="2:15" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B4" s="12">
         <v>2011</v>
       </c>
       <c r="C4" s="13" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D4" s="13" t="s">
-        <v>33</v>
-      </c>
-      <c r="E4" s="14" t="s">
-        <v>11</v>
-      </c>
-      <c r="F4" s="14"/>
-      <c r="G4" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="H4" s="14">
-        <v>192</v>
-      </c>
-      <c r="I4" s="14"/>
-      <c r="J4" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="K4" s="26">
+        <v>29</v>
+      </c>
+      <c r="E4" s="46" t="s">
+        <v>10</v>
+      </c>
+      <c r="F4" s="46" t="s">
+        <v>126</v>
+      </c>
+      <c r="G4" s="46" t="s">
+        <v>124</v>
+      </c>
+      <c r="H4" s="46">
+        <v>253</v>
+      </c>
+      <c r="I4" s="47" t="s">
+        <v>15</v>
+      </c>
+      <c r="J4" s="47">
         <v>2</v>
       </c>
-      <c r="L4" s="2"/>
-      <c r="M4" s="14"/>
-    </row>
-    <row r="5" spans="2:13" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="K4" s="2"/>
+      <c r="L4" s="14"/>
+      <c r="O4" s="46"/>
+    </row>
+    <row r="5" spans="2:15" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="12">
         <v>2012</v>
       </c>
       <c r="C5" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="D5" s="13" t="s">
+        <v>44</v>
+      </c>
+      <c r="E5" s="46" t="s">
         <v>10</v>
       </c>
-      <c r="D5" s="13" t="s">
-        <v>48</v>
-      </c>
-      <c r="E5" s="14" t="s">
-        <v>11</v>
-      </c>
-      <c r="F5" s="14"/>
-      <c r="G5" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="H5" s="14">
-        <v>192</v>
-      </c>
-      <c r="I5" s="14">
+      <c r="F5" s="46" t="s">
+        <v>126</v>
+      </c>
+      <c r="G5" s="46" t="s">
+        <v>124</v>
+      </c>
+      <c r="H5" s="46">
         <v>263</v>
       </c>
-      <c r="J5" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="K5" s="26">
+      <c r="I5" s="47" t="s">
+        <v>15</v>
+      </c>
+      <c r="J5" s="47">
         <v>1</v>
       </c>
-      <c r="L5" s="2"/>
-      <c r="M5" s="14"/>
-    </row>
-    <row r="6" spans="2:13" ht="50.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="K5" s="2"/>
+      <c r="L5" s="14"/>
+      <c r="O5" s="46"/>
+    </row>
+    <row r="6" spans="2:15" ht="50.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6" s="12">
         <v>2013</v>
       </c>
       <c r="C6" s="13" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D6" s="13" t="s">
-        <v>49</v>
-      </c>
-      <c r="E6" s="14" t="s">
-        <v>12</v>
-      </c>
-      <c r="F6" s="14"/>
-      <c r="G6" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="H6" s="14">
-        <v>192</v>
-      </c>
-      <c r="I6" s="14">
+        <v>45</v>
+      </c>
+      <c r="E6" s="46" t="s">
+        <v>11</v>
+      </c>
+      <c r="F6" s="46" t="s">
+        <v>126</v>
+      </c>
+      <c r="G6" s="46" t="s">
+        <v>124</v>
+      </c>
+      <c r="H6" s="46">
         <v>293</v>
       </c>
-      <c r="J6" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="K6" s="2">
+      <c r="I6" s="47" t="s">
+        <v>15</v>
+      </c>
+      <c r="J6" s="47">
         <v>2</v>
       </c>
-      <c r="L6" s="2"/>
-      <c r="M6" s="14"/>
-    </row>
-    <row r="7" spans="2:13" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="K6" s="2"/>
+      <c r="L6" s="14"/>
+      <c r="O6" s="46"/>
+    </row>
+    <row r="7" spans="2:15" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="12">
         <v>2015</v>
       </c>
       <c r="C7" s="13" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D7" s="13" t="s">
-        <v>46</v>
-      </c>
-      <c r="E7" s="14" t="s">
-        <v>13</v>
-      </c>
-      <c r="F7" s="14"/>
-      <c r="G7" s="14" t="s">
-        <v>26</v>
-      </c>
-      <c r="H7" s="14">
-        <v>500</v>
-      </c>
-      <c r="I7" s="14"/>
-      <c r="J7" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="K7" s="2">
+        <v>42</v>
+      </c>
+      <c r="E7" s="46" t="s">
+        <v>12</v>
+      </c>
+      <c r="F7" s="46" t="s">
+        <v>127</v>
+      </c>
+      <c r="G7" s="46" t="s">
+        <v>125</v>
+      </c>
+      <c r="H7" s="46"/>
+      <c r="I7" s="47" t="s">
+        <v>15</v>
+      </c>
+      <c r="J7" s="47">
         <v>2</v>
       </c>
-      <c r="L7" s="2"/>
-      <c r="M7" s="14"/>
-    </row>
-    <row r="8" spans="2:13" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="K7" s="2"/>
+      <c r="L7" s="14"/>
+      <c r="O7" s="46"/>
+    </row>
+    <row r="8" spans="2:15" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B8" s="12">
         <v>2016</v>
       </c>
       <c r="C8" s="13" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D8" s="13" t="s">
-        <v>45</v>
-      </c>
-      <c r="E8" s="14" t="s">
-        <v>13</v>
-      </c>
-      <c r="F8" s="14"/>
-      <c r="G8" s="14" t="s">
-        <v>26</v>
-      </c>
-      <c r="H8" s="14">
-        <v>500</v>
-      </c>
-      <c r="I8" s="14">
+        <v>41</v>
+      </c>
+      <c r="E8" s="46" t="s">
+        <v>12</v>
+      </c>
+      <c r="F8" s="46" t="s">
+        <v>127</v>
+      </c>
+      <c r="G8" s="46" t="s">
+        <v>125</v>
+      </c>
+      <c r="H8" s="46">
         <v>350</v>
       </c>
-      <c r="J8" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="K8" s="2">
+      <c r="I8" s="47" t="s">
+        <v>15</v>
+      </c>
+      <c r="J8" s="47">
         <v>1</v>
       </c>
-      <c r="L8" s="2"/>
-      <c r="M8" s="14"/>
-    </row>
-    <row r="9" spans="2:13" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="K8" s="2"/>
+      <c r="L8" s="14"/>
+      <c r="O8" s="46"/>
+    </row>
+    <row r="9" spans="2:15" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B9" s="12">
         <v>2017</v>
       </c>
       <c r="C9" s="13" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D9" s="13" t="s">
-        <v>122</v>
-      </c>
-      <c r="E9" s="14" t="s">
-        <v>13</v>
-      </c>
-      <c r="F9" s="14"/>
-      <c r="G9" s="14" t="s">
-        <v>26</v>
-      </c>
-      <c r="H9" s="14">
-        <v>500</v>
-      </c>
-      <c r="I9" s="14">
+        <v>118</v>
+      </c>
+      <c r="E9" s="46" t="s">
+        <v>12</v>
+      </c>
+      <c r="F9" s="46" t="s">
+        <v>127</v>
+      </c>
+      <c r="G9" s="46" t="s">
+        <v>125</v>
+      </c>
+      <c r="H9" s="46">
         <v>1743</v>
       </c>
-      <c r="J9" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="K9" s="2" t="s">
-        <v>123</v>
-      </c>
-      <c r="L9" s="2"/>
-      <c r="M9" s="14"/>
-    </row>
-    <row r="10" spans="2:13" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="I9" s="47" t="s">
+        <v>17</v>
+      </c>
+      <c r="J9" s="47" t="s">
+        <v>119</v>
+      </c>
+      <c r="K9" s="2"/>
+      <c r="L9" s="14"/>
+      <c r="O9" s="46"/>
+    </row>
+    <row r="10" spans="2:15" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B10" s="12">
         <v>2018</v>
       </c>
       <c r="C10" s="13" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D10" s="13" t="s">
-        <v>44</v>
-      </c>
-      <c r="E10" s="14" t="s">
-        <v>13</v>
-      </c>
-      <c r="F10" s="14"/>
-      <c r="G10" s="14" t="s">
-        <v>26</v>
-      </c>
-      <c r="H10" s="14">
-        <v>500</v>
-      </c>
-      <c r="I10" s="14"/>
-      <c r="J10" s="2" t="s">
-        <v>20</v>
-      </c>
+        <v>40</v>
+      </c>
+      <c r="E10" s="46" t="s">
+        <v>12</v>
+      </c>
+      <c r="F10" s="46" t="s">
+        <v>127</v>
+      </c>
+      <c r="G10" s="46" t="s">
+        <v>125</v>
+      </c>
+      <c r="H10" s="46"/>
+      <c r="I10" s="47" t="s">
+        <v>18</v>
+      </c>
+      <c r="J10" s="47"/>
       <c r="K10" s="2"/>
-      <c r="L10" s="2"/>
-      <c r="M10" s="14"/>
-    </row>
-    <row r="11" spans="2:13" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="L10" s="14"/>
+      <c r="O10" s="46"/>
+    </row>
+    <row r="11" spans="2:15" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B11" s="12">
         <v>2019</v>
       </c>
       <c r="C11" s="13" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D11" s="13" t="s">
-        <v>43</v>
-      </c>
-      <c r="E11" s="14" t="s">
-        <v>13</v>
-      </c>
-      <c r="F11" s="14"/>
-      <c r="G11" s="14" t="s">
-        <v>26</v>
-      </c>
-      <c r="H11" s="14">
-        <v>500</v>
-      </c>
-      <c r="I11" s="14"/>
-      <c r="J11" s="2" t="s">
-        <v>20</v>
-      </c>
+        <v>39</v>
+      </c>
+      <c r="E11" s="46" t="s">
+        <v>12</v>
+      </c>
+      <c r="F11" s="46" t="s">
+        <v>127</v>
+      </c>
+      <c r="G11" s="46" t="s">
+        <v>125</v>
+      </c>
+      <c r="H11" s="46"/>
+      <c r="I11" s="47" t="s">
+        <v>18</v>
+      </c>
+      <c r="J11" s="47"/>
       <c r="K11" s="2"/>
-      <c r="L11" s="2"/>
-      <c r="M11" s="14"/>
-    </row>
-    <row r="12" spans="2:13" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="L11" s="14"/>
+      <c r="O11" s="46"/>
+    </row>
+    <row r="12" spans="2:15" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B12" s="12">
         <v>2020</v>
       </c>
       <c r="C12" s="13" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D12" s="13" t="s">
-        <v>42</v>
-      </c>
-      <c r="E12" s="14" t="s">
-        <v>13</v>
-      </c>
-      <c r="F12" s="14"/>
-      <c r="G12" s="14" t="s">
-        <v>26</v>
-      </c>
-      <c r="H12" s="14">
-        <v>500</v>
-      </c>
-      <c r="I12" s="14"/>
-      <c r="J12" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="K12" s="2">
+        <v>38</v>
+      </c>
+      <c r="E12" s="46" t="s">
+        <v>12</v>
+      </c>
+      <c r="F12" s="46" t="s">
+        <v>127</v>
+      </c>
+      <c r="G12" s="46" t="s">
+        <v>125</v>
+      </c>
+      <c r="H12" s="46"/>
+      <c r="I12" s="47" t="s">
+        <v>18</v>
+      </c>
+      <c r="J12" s="47">
         <v>4</v>
       </c>
-      <c r="L12" s="2"/>
-      <c r="M12" s="14"/>
-    </row>
-    <row r="13" spans="2:13" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="K12" s="2"/>
+      <c r="L12" s="14"/>
+      <c r="O12" s="46"/>
+    </row>
+    <row r="13" spans="2:15" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B13" s="12">
         <v>2021</v>
       </c>
       <c r="C13" s="13" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D13" s="13" t="s">
-        <v>41</v>
-      </c>
-      <c r="E13" s="14" t="s">
-        <v>13</v>
-      </c>
-      <c r="F13" s="14"/>
-      <c r="G13" s="14" t="s">
-        <v>26</v>
-      </c>
-      <c r="H13" s="14">
-        <v>500</v>
-      </c>
-      <c r="I13" s="14"/>
-      <c r="J13" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="K13" s="2">
+        <v>37</v>
+      </c>
+      <c r="E13" s="46" t="s">
+        <v>12</v>
+      </c>
+      <c r="F13" s="46" t="s">
+        <v>127</v>
+      </c>
+      <c r="G13" s="46" t="s">
+        <v>125</v>
+      </c>
+      <c r="H13" s="46"/>
+      <c r="I13" s="47" t="s">
+        <v>18</v>
+      </c>
+      <c r="J13" s="47">
         <v>9</v>
       </c>
-      <c r="L13" s="2"/>
-      <c r="M13" s="14"/>
-    </row>
-    <row r="14" spans="2:13" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="K13" s="2"/>
+      <c r="L13" s="14"/>
+      <c r="O13" s="46"/>
+    </row>
+    <row r="14" spans="2:15" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B14" s="12">
         <v>2023</v>
       </c>
       <c r="C14" s="13" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D14" s="13" t="s">
-        <v>40</v>
-      </c>
-      <c r="E14" s="14" t="s">
-        <v>13</v>
-      </c>
-      <c r="F14" s="14"/>
-      <c r="G14" s="14" t="s">
-        <v>26</v>
-      </c>
-      <c r="H14" s="14">
-        <v>500</v>
-      </c>
-      <c r="I14" s="14"/>
-      <c r="J14" s="2" t="s">
-        <v>21</v>
-      </c>
+        <v>36</v>
+      </c>
+      <c r="E14" s="46" t="s">
+        <v>12</v>
+      </c>
+      <c r="F14" s="46" t="s">
+        <v>127</v>
+      </c>
+      <c r="G14" s="46" t="s">
+        <v>125</v>
+      </c>
+      <c r="H14" s="46"/>
+      <c r="I14" s="47" t="s">
+        <v>19</v>
+      </c>
+      <c r="J14" s="47"/>
       <c r="K14" s="2"/>
-      <c r="L14" s="2"/>
-      <c r="M14" s="14"/>
-    </row>
-    <row r="15" spans="2:13" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="L14" s="14"/>
+      <c r="O14" s="46"/>
+    </row>
+    <row r="15" spans="2:15" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B15" s="12">
         <v>2024</v>
       </c>
       <c r="C15" s="13" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D15" s="13" t="s">
-        <v>39</v>
-      </c>
-      <c r="E15" s="14" t="s">
-        <v>13</v>
-      </c>
-      <c r="F15" s="14"/>
-      <c r="G15" s="14" t="s">
-        <v>26</v>
-      </c>
-      <c r="H15" s="14">
-        <v>500</v>
-      </c>
-      <c r="I15" s="14"/>
-      <c r="J15" s="2" t="s">
-        <v>21</v>
-      </c>
+        <v>35</v>
+      </c>
+      <c r="E15" s="46" t="s">
+        <v>12</v>
+      </c>
+      <c r="F15" s="46" t="s">
+        <v>127</v>
+      </c>
+      <c r="G15" s="46" t="s">
+        <v>125</v>
+      </c>
+      <c r="H15" s="46"/>
+      <c r="I15" s="47" t="s">
+        <v>19</v>
+      </c>
+      <c r="J15" s="47"/>
       <c r="K15" s="2"/>
-      <c r="L15" s="2"/>
-      <c r="M15" s="14"/>
+      <c r="L15" s="14"/>
+      <c r="O15" s="46"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="8" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
+  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -2046,26 +2114,26 @@
         <v>0</v>
       </c>
       <c r="C3" s="18" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="D3" s="18" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="E3" s="18" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="F3" s="18" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="G3" s="18" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="H3" s="18" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="I3" s="16"/>
       <c r="J3" s="16" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="L3" s="15"/>
     </row>
@@ -2171,7 +2239,7 @@
     <row r="7" spans="2:12" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
     <row r="9" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B9" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="C9">
         <f>SUM(C4:C6)</f>
@@ -2196,7 +2264,7 @@
     </row>
     <row r="12" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B12" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="D12">
         <f>C9-D9</f>
@@ -2205,26 +2273,26 @@
     </row>
     <row r="14" spans="2:12" x14ac:dyDescent="0.3">
       <c r="C14" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17" s="21" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B18" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="C18" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="D18" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="E18" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.3">
@@ -2274,7 +2342,7 @@
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A22" s="21" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="B22" s="21">
         <f>SUM(B19:B21)</f>
@@ -2292,7 +2360,7 @@
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="B24">
         <f>1068-755</f>
@@ -2301,7 +2369,7 @@
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="B25">
         <f>755-212</f>
@@ -2310,7 +2378,7 @@
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A26" s="21" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="B26" s="21">
         <f>B24+B25</f>
@@ -2319,7 +2387,7 @@
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A28" s="21" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="B28" s="22">
         <f>B26/B22</f>
@@ -2328,7 +2396,7 @@
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A30" s="21" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="B30" s="20">
         <f>AVERAGE(E19:E21)</f>
@@ -2337,7 +2405,7 @@
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="B31" s="20">
         <f>MEDIAN(E19:E21)</f>
@@ -2363,20 +2431,20 @@
   </cols>
   <sheetData>
     <row r="3" spans="2:7" ht="26.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="C3" s="27"/>
-      <c r="D3" s="27"/>
-      <c r="E3" s="27"/>
+      <c r="C3" s="45"/>
+      <c r="D3" s="45"/>
+      <c r="E3" s="45"/>
     </row>
     <row r="4" spans="2:7" ht="56.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B4" s="4"/>
       <c r="C4" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="E4" s="5" t="s">
         <v>22</v>
-      </c>
-      <c r="D4" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="E4" s="5" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="5" spans="2:7" ht="26.25" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
code update, table update
Created total acoustic hours to get recording effort. Updated table with hours.
</commit_message>
<xml_diff>
--- a/manuscript/BANTER_Pseudorca-AllTablesxlsx.xlsx
+++ b/manuscript/BANTER_Pseudorca-AllTablesxlsx.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yvonne.barkley\Github\BANTER_Pseudorca\manuscript\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37A33E58-30D1-43E4-8D29-ABDD14ED5008}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCDA9BBB-A165-4AB8-8CEB-C8BF30F2BEF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="4140" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Threshold_Table" sheetId="4" r:id="rId1"/>
@@ -145,9 +145,6 @@
     <t>Visually Verified Pc</t>
   </si>
   <si>
-    <t>Total Acoustic Hours</t>
-  </si>
-  <si>
     <t>Total Events</t>
   </si>
   <si>
@@ -458,6 +455,9 @@
   </si>
   <si>
     <t>2 – 85 kHz</t>
+  </si>
+  <si>
+    <t>Total Recording Hours</t>
   </si>
 </sst>
 </file>
@@ -970,14 +970,14 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1272,7 +1272,7 @@
     <row r="2" spans="2:18" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
       <c r="B2" s="26"/>
       <c r="C2" s="27" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D2" s="28"/>
       <c r="E2" s="28"/>
@@ -1292,7 +1292,7 @@
     </row>
     <row r="3" spans="2:18" ht="42" x14ac:dyDescent="0.4">
       <c r="B3" s="44" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C3" s="33">
         <v>2017</v>
@@ -1313,7 +1313,7 @@
       <c r="M3" s="30"/>
       <c r="N3" s="32"/>
       <c r="O3" s="33" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="P3" s="30"/>
       <c r="Q3" s="30"/>
@@ -1322,52 +1322,52 @@
     <row r="4" spans="2:18" ht="21" x14ac:dyDescent="0.4">
       <c r="B4" s="35"/>
       <c r="C4" s="36" t="s">
+        <v>58</v>
+      </c>
+      <c r="D4" s="37" t="s">
         <v>59</v>
       </c>
-      <c r="D4" s="37" t="s">
+      <c r="E4" s="37" t="s">
         <v>60</v>
       </c>
-      <c r="E4" s="37" t="s">
+      <c r="F4" s="38" t="s">
+        <v>120</v>
+      </c>
+      <c r="G4" s="36" t="s">
         <v>61</v>
       </c>
-      <c r="F4" s="38" t="s">
-        <v>121</v>
-      </c>
-      <c r="G4" s="36" t="s">
-        <v>62</v>
-      </c>
       <c r="H4" s="37" t="s">
+        <v>59</v>
+      </c>
+      <c r="I4" s="37" t="s">
         <v>60</v>
       </c>
-      <c r="I4" s="37" t="s">
+      <c r="J4" s="38" t="s">
+        <v>120</v>
+      </c>
+      <c r="K4" s="36" t="s">
         <v>61</v>
       </c>
-      <c r="J4" s="38" t="s">
-        <v>121</v>
-      </c>
-      <c r="K4" s="36" t="s">
-        <v>62</v>
-      </c>
       <c r="L4" s="37" t="s">
+        <v>59</v>
+      </c>
+      <c r="M4" s="37" t="s">
         <v>60</v>
       </c>
-      <c r="M4" s="37" t="s">
+      <c r="N4" s="38" t="s">
+        <v>120</v>
+      </c>
+      <c r="O4" s="36" t="s">
         <v>61</v>
       </c>
-      <c r="N4" s="38" t="s">
-        <v>121</v>
-      </c>
-      <c r="O4" s="36" t="s">
-        <v>62</v>
-      </c>
       <c r="P4" s="37" t="s">
+        <v>59</v>
+      </c>
+      <c r="Q4" s="37" t="s">
         <v>60</v>
       </c>
-      <c r="Q4" s="37" t="s">
-        <v>61</v>
-      </c>
       <c r="R4" s="38" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="5" spans="2:18" ht="21" x14ac:dyDescent="0.4">
@@ -1375,52 +1375,52 @@
         <v>0.5</v>
       </c>
       <c r="C5" s="36" t="s">
+        <v>62</v>
+      </c>
+      <c r="D5" s="37" t="s">
         <v>63</v>
       </c>
-      <c r="D5" s="37" t="s">
+      <c r="E5" s="37" t="s">
         <v>64</v>
       </c>
-      <c r="E5" s="37" t="s">
+      <c r="F5" s="38" t="s">
         <v>65</v>
       </c>
-      <c r="F5" s="38" t="s">
+      <c r="G5" s="36" t="s">
         <v>66</v>
       </c>
-      <c r="G5" s="36" t="s">
+      <c r="H5" s="37" t="s">
         <v>67</v>
       </c>
-      <c r="H5" s="37" t="s">
+      <c r="I5" s="37" t="s">
         <v>68</v>
       </c>
-      <c r="I5" s="37" t="s">
+      <c r="J5" s="38" t="s">
         <v>69</v>
       </c>
-      <c r="J5" s="38" t="s">
+      <c r="K5" s="36" t="s">
         <v>70</v>
       </c>
-      <c r="K5" s="36" t="s">
+      <c r="L5" s="37" t="s">
         <v>71</v>
       </c>
-      <c r="L5" s="37" t="s">
+      <c r="M5" s="37" t="s">
         <v>72</v>
       </c>
-      <c r="M5" s="37" t="s">
+      <c r="N5" s="38" t="s">
         <v>73</v>
       </c>
-      <c r="N5" s="38" t="s">
+      <c r="O5" s="36" t="s">
         <v>74</v>
       </c>
-      <c r="O5" s="36" t="s">
+      <c r="P5" s="37" t="s">
         <v>75</v>
       </c>
-      <c r="P5" s="37" t="s">
+      <c r="Q5" s="37" t="s">
         <v>76</v>
       </c>
-      <c r="Q5" s="37" t="s">
+      <c r="R5" s="38" t="s">
         <v>77</v>
-      </c>
-      <c r="R5" s="38" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="6" spans="2:18" ht="21" x14ac:dyDescent="0.4">
@@ -1428,52 +1428,52 @@
         <v>0.6</v>
       </c>
       <c r="C6" s="36" t="s">
+        <v>78</v>
+      </c>
+      <c r="D6" s="37" t="s">
         <v>79</v>
       </c>
-      <c r="D6" s="37" t="s">
+      <c r="E6" s="37" t="s">
         <v>80</v>
       </c>
-      <c r="E6" s="37" t="s">
+      <c r="F6" s="38" t="s">
+        <v>65</v>
+      </c>
+      <c r="G6" s="36" t="s">
         <v>81</v>
       </c>
-      <c r="F6" s="38" t="s">
-        <v>66</v>
-      </c>
-      <c r="G6" s="36" t="s">
+      <c r="H6" s="37" t="s">
         <v>82</v>
       </c>
-      <c r="H6" s="37" t="s">
+      <c r="I6" s="37" t="s">
         <v>83</v>
       </c>
-      <c r="I6" s="37" t="s">
+      <c r="J6" s="38" t="s">
+        <v>73</v>
+      </c>
+      <c r="K6" s="36" t="s">
         <v>84</v>
       </c>
-      <c r="J6" s="38" t="s">
-        <v>74</v>
-      </c>
-      <c r="K6" s="36" t="s">
+      <c r="L6" s="37" t="s">
         <v>85</v>
       </c>
-      <c r="L6" s="37" t="s">
+      <c r="M6" s="37" t="s">
+        <v>84</v>
+      </c>
+      <c r="N6" s="38" t="s">
+        <v>85</v>
+      </c>
+      <c r="O6" s="36" t="s">
+        <v>76</v>
+      </c>
+      <c r="P6" s="37" t="s">
         <v>86</v>
       </c>
-      <c r="M6" s="37" t="s">
-        <v>85</v>
-      </c>
-      <c r="N6" s="38" t="s">
-        <v>86</v>
-      </c>
-      <c r="O6" s="36" t="s">
-        <v>77</v>
-      </c>
-      <c r="P6" s="37" t="s">
+      <c r="Q6" s="37" t="s">
         <v>87</v>
       </c>
-      <c r="Q6" s="37" t="s">
+      <c r="R6" s="38" t="s">
         <v>88</v>
-      </c>
-      <c r="R6" s="38" t="s">
-        <v>89</v>
       </c>
     </row>
     <row r="7" spans="2:18" ht="21" x14ac:dyDescent="0.4">
@@ -1481,52 +1481,52 @@
         <v>0.7</v>
       </c>
       <c r="C7" s="36" t="s">
+        <v>89</v>
+      </c>
+      <c r="D7" s="37" t="s">
         <v>90</v>
       </c>
-      <c r="D7" s="37" t="s">
+      <c r="E7" s="37" t="s">
         <v>91</v>
       </c>
-      <c r="E7" s="37" t="s">
+      <c r="F7" s="38" t="s">
         <v>92</v>
       </c>
-      <c r="F7" s="38" t="s">
+      <c r="G7" s="36" t="s">
         <v>93</v>
       </c>
-      <c r="G7" s="36" t="s">
+      <c r="H7" s="37" t="s">
         <v>94</v>
       </c>
-      <c r="H7" s="37" t="s">
+      <c r="I7" s="37" t="s">
         <v>95</v>
       </c>
-      <c r="I7" s="37" t="s">
+      <c r="J7" s="38" t="s">
         <v>96</v>
       </c>
-      <c r="J7" s="38" t="s">
+      <c r="K7" s="36" t="s">
         <v>97</v>
       </c>
-      <c r="K7" s="36" t="s">
+      <c r="L7" s="37" t="s">
+        <v>96</v>
+      </c>
+      <c r="M7" s="37" t="s">
+        <v>97</v>
+      </c>
+      <c r="N7" s="38" t="s">
+        <v>96</v>
+      </c>
+      <c r="O7" s="36" t="s">
         <v>98</v>
       </c>
-      <c r="L7" s="37" t="s">
-        <v>97</v>
-      </c>
-      <c r="M7" s="37" t="s">
-        <v>98</v>
-      </c>
-      <c r="N7" s="38" t="s">
-        <v>97</v>
-      </c>
-      <c r="O7" s="36" t="s">
+      <c r="P7" s="37" t="s">
         <v>99</v>
       </c>
-      <c r="P7" s="37" t="s">
+      <c r="Q7" s="37" t="s">
         <v>100</v>
       </c>
-      <c r="Q7" s="37" t="s">
+      <c r="R7" s="38" t="s">
         <v>101</v>
-      </c>
-      <c r="R7" s="38" t="s">
-        <v>102</v>
       </c>
     </row>
     <row r="8" spans="2:18" ht="21" x14ac:dyDescent="0.4">
@@ -1534,52 +1534,52 @@
         <v>0.8</v>
       </c>
       <c r="C8" s="36" t="s">
+        <v>102</v>
+      </c>
+      <c r="D8" s="37" t="s">
         <v>103</v>
       </c>
-      <c r="D8" s="37" t="s">
+      <c r="E8" s="37" t="s">
+        <v>102</v>
+      </c>
+      <c r="F8" s="38" t="s">
+        <v>103</v>
+      </c>
+      <c r="G8" s="36" t="s">
         <v>104</v>
       </c>
-      <c r="E8" s="37" t="s">
-        <v>103</v>
-      </c>
-      <c r="F8" s="38" t="s">
-        <v>104</v>
-      </c>
-      <c r="G8" s="36" t="s">
+      <c r="H8" s="37" t="s">
         <v>105</v>
       </c>
-      <c r="H8" s="37" t="s">
+      <c r="I8" s="37" t="s">
+        <v>105</v>
+      </c>
+      <c r="J8" s="38" t="s">
         <v>106</v>
       </c>
-      <c r="I8" s="37" t="s">
-        <v>106</v>
-      </c>
-      <c r="J8" s="38" t="s">
+      <c r="K8" s="36" t="s">
         <v>107</v>
       </c>
-      <c r="K8" s="36" t="s">
+      <c r="L8" s="37" t="s">
+        <v>107</v>
+      </c>
+      <c r="M8" s="37" t="s">
+        <v>107</v>
+      </c>
+      <c r="N8" s="38" t="s">
+        <v>107</v>
+      </c>
+      <c r="O8" s="36" t="s">
         <v>108</v>
       </c>
-      <c r="L8" s="37" t="s">
-        <v>108</v>
-      </c>
-      <c r="M8" s="37" t="s">
-        <v>108</v>
-      </c>
-      <c r="N8" s="38" t="s">
-        <v>108</v>
-      </c>
-      <c r="O8" s="36" t="s">
+      <c r="P8" s="37" t="s">
         <v>109</v>
       </c>
-      <c r="P8" s="37" t="s">
+      <c r="Q8" s="37" t="s">
         <v>110</v>
       </c>
-      <c r="Q8" s="37" t="s">
+      <c r="R8" s="38" t="s">
         <v>111</v>
-      </c>
-      <c r="R8" s="38" t="s">
-        <v>112</v>
       </c>
     </row>
     <row r="9" spans="2:18" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
@@ -1587,57 +1587,57 @@
         <v>0.9</v>
       </c>
       <c r="C9" s="41" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D9" s="42" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E9" s="42" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="F9" s="43" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="G9" s="41" t="s">
+        <v>112</v>
+      </c>
+      <c r="H9" s="42" t="s">
+        <v>112</v>
+      </c>
+      <c r="I9" s="42" t="s">
+        <v>112</v>
+      </c>
+      <c r="J9" s="43" t="s">
+        <v>112</v>
+      </c>
+      <c r="K9" s="41" t="s">
+        <v>112</v>
+      </c>
+      <c r="L9" s="42" t="s">
+        <v>112</v>
+      </c>
+      <c r="M9" s="42" t="s">
+        <v>112</v>
+      </c>
+      <c r="N9" s="43" t="s">
+        <v>112</v>
+      </c>
+      <c r="O9" s="41" t="s">
         <v>113</v>
       </c>
-      <c r="H9" s="42" t="s">
+      <c r="P9" s="42" t="s">
         <v>113</v>
       </c>
-      <c r="I9" s="42" t="s">
+      <c r="Q9" s="42" t="s">
         <v>113</v>
       </c>
-      <c r="J9" s="43" t="s">
+      <c r="R9" s="43" t="s">
         <v>113</v>
-      </c>
-      <c r="K9" s="41" t="s">
-        <v>113</v>
-      </c>
-      <c r="L9" s="42" t="s">
-        <v>113</v>
-      </c>
-      <c r="M9" s="42" t="s">
-        <v>113</v>
-      </c>
-      <c r="N9" s="43" t="s">
-        <v>113</v>
-      </c>
-      <c r="O9" s="41" t="s">
-        <v>114</v>
-      </c>
-      <c r="P9" s="42" t="s">
-        <v>114</v>
-      </c>
-      <c r="Q9" s="42" t="s">
-        <v>114</v>
-      </c>
-      <c r="R9" s="43" t="s">
-        <v>114</v>
       </c>
     </row>
     <row r="14" spans="2:18" x14ac:dyDescent="0.3">
       <c r="C14" s="24" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
   </sheetData>
@@ -1665,7 +1665,7 @@
         <v>1</v>
       </c>
       <c r="D2" s="12" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E2" s="12" t="s">
         <v>2</v>
@@ -1674,22 +1674,22 @@
         <v>14</v>
       </c>
       <c r="G2" s="12" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="H2" s="12" t="s">
-        <v>23</v>
+        <v>127</v>
       </c>
       <c r="I2" s="12" t="s">
         <v>16</v>
       </c>
       <c r="J2" s="12" t="s">
+        <v>114</v>
+      </c>
+      <c r="K2" s="12" t="s">
         <v>115</v>
       </c>
-      <c r="K2" s="12" t="s">
-        <v>116</v>
-      </c>
       <c r="L2" s="12" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="O2" s="25" t="s">
         <v>3</v>
@@ -1703,29 +1703,29 @@
         <v>4</v>
       </c>
       <c r="D3" s="13" t="s">
-        <v>43</v>
-      </c>
-      <c r="E3" s="46" t="s">
+        <v>42</v>
+      </c>
+      <c r="E3" s="45" t="s">
         <v>10</v>
       </c>
-      <c r="F3" s="46" t="s">
-        <v>126</v>
-      </c>
-      <c r="G3" s="46" t="s">
-        <v>124</v>
-      </c>
-      <c r="H3" s="46">
+      <c r="F3" s="45" t="s">
+        <v>125</v>
+      </c>
+      <c r="G3" s="45" t="s">
+        <v>123</v>
+      </c>
+      <c r="H3" s="45">
         <v>1445</v>
       </c>
-      <c r="I3" s="47" t="s">
+      <c r="I3" s="46" t="s">
         <v>15</v>
       </c>
-      <c r="J3" s="47" t="s">
-        <v>117</v>
+      <c r="J3" s="46" t="s">
+        <v>116</v>
       </c>
       <c r="K3" s="2"/>
       <c r="L3" s="14"/>
-      <c r="O3" s="46"/>
+      <c r="O3" s="45"/>
     </row>
     <row r="4" spans="2:15" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B4" s="12">
@@ -1735,29 +1735,29 @@
         <v>8</v>
       </c>
       <c r="D4" s="13" t="s">
-        <v>29</v>
-      </c>
-      <c r="E4" s="46" t="s">
+        <v>28</v>
+      </c>
+      <c r="E4" s="45" t="s">
         <v>10</v>
       </c>
-      <c r="F4" s="46" t="s">
-        <v>126</v>
-      </c>
-      <c r="G4" s="46" t="s">
-        <v>124</v>
-      </c>
-      <c r="H4" s="46">
+      <c r="F4" s="45" t="s">
+        <v>125</v>
+      </c>
+      <c r="G4" s="45" t="s">
+        <v>123</v>
+      </c>
+      <c r="H4" s="45">
         <v>253</v>
       </c>
-      <c r="I4" s="47" t="s">
+      <c r="I4" s="46" t="s">
         <v>15</v>
       </c>
-      <c r="J4" s="47">
+      <c r="J4" s="46">
         <v>2</v>
       </c>
       <c r="K4" s="2"/>
       <c r="L4" s="14"/>
-      <c r="O4" s="46"/>
+      <c r="O4" s="45"/>
     </row>
     <row r="5" spans="2:15" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="12">
@@ -1767,29 +1767,29 @@
         <v>9</v>
       </c>
       <c r="D5" s="13" t="s">
-        <v>44</v>
-      </c>
-      <c r="E5" s="46" t="s">
+        <v>43</v>
+      </c>
+      <c r="E5" s="45" t="s">
         <v>10</v>
       </c>
-      <c r="F5" s="46" t="s">
-        <v>126</v>
-      </c>
-      <c r="G5" s="46" t="s">
-        <v>124</v>
-      </c>
-      <c r="H5" s="46">
+      <c r="F5" s="45" t="s">
+        <v>125</v>
+      </c>
+      <c r="G5" s="45" t="s">
+        <v>123</v>
+      </c>
+      <c r="H5" s="45">
         <v>263</v>
       </c>
-      <c r="I5" s="47" t="s">
+      <c r="I5" s="46" t="s">
         <v>15</v>
       </c>
-      <c r="J5" s="47">
+      <c r="J5" s="46">
         <v>1</v>
       </c>
       <c r="K5" s="2"/>
       <c r="L5" s="14"/>
-      <c r="O5" s="46"/>
+      <c r="O5" s="45"/>
     </row>
     <row r="6" spans="2:15" ht="50.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6" s="12">
@@ -1799,29 +1799,29 @@
         <v>13</v>
       </c>
       <c r="D6" s="13" t="s">
-        <v>45</v>
-      </c>
-      <c r="E6" s="46" t="s">
+        <v>44</v>
+      </c>
+      <c r="E6" s="45" t="s">
         <v>11</v>
       </c>
-      <c r="F6" s="46" t="s">
-        <v>126</v>
-      </c>
-      <c r="G6" s="46" t="s">
-        <v>124</v>
-      </c>
-      <c r="H6" s="46">
+      <c r="F6" s="45" t="s">
+        <v>125</v>
+      </c>
+      <c r="G6" s="45" t="s">
+        <v>123</v>
+      </c>
+      <c r="H6" s="45">
         <v>293</v>
       </c>
-      <c r="I6" s="47" t="s">
+      <c r="I6" s="46" t="s">
         <v>15</v>
       </c>
-      <c r="J6" s="47">
+      <c r="J6" s="46">
         <v>2</v>
       </c>
       <c r="K6" s="2"/>
       <c r="L6" s="14"/>
-      <c r="O6" s="46"/>
+      <c r="O6" s="45"/>
     </row>
     <row r="7" spans="2:15" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="12">
@@ -1831,27 +1831,29 @@
         <v>6</v>
       </c>
       <c r="D7" s="13" t="s">
-        <v>42</v>
-      </c>
-      <c r="E7" s="46" t="s">
+        <v>41</v>
+      </c>
+      <c r="E7" s="45" t="s">
         <v>12</v>
       </c>
-      <c r="F7" s="46" t="s">
-        <v>127</v>
-      </c>
-      <c r="G7" s="46" t="s">
-        <v>125</v>
-      </c>
-      <c r="H7" s="46"/>
-      <c r="I7" s="47" t="s">
+      <c r="F7" s="45" t="s">
+        <v>126</v>
+      </c>
+      <c r="G7" s="45" t="s">
+        <v>124</v>
+      </c>
+      <c r="H7" s="45">
+        <v>306</v>
+      </c>
+      <c r="I7" s="46" t="s">
         <v>15</v>
       </c>
-      <c r="J7" s="47">
+      <c r="J7" s="46">
         <v>2</v>
       </c>
       <c r="K7" s="2"/>
       <c r="L7" s="14"/>
-      <c r="O7" s="46"/>
+      <c r="O7" s="45"/>
     </row>
     <row r="8" spans="2:15" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B8" s="12">
@@ -1861,29 +1863,29 @@
         <v>5</v>
       </c>
       <c r="D8" s="13" t="s">
-        <v>41</v>
-      </c>
-      <c r="E8" s="46" t="s">
+        <v>40</v>
+      </c>
+      <c r="E8" s="45" t="s">
         <v>12</v>
       </c>
-      <c r="F8" s="46" t="s">
-        <v>127</v>
-      </c>
-      <c r="G8" s="46" t="s">
-        <v>125</v>
-      </c>
-      <c r="H8" s="46">
+      <c r="F8" s="45" t="s">
+        <v>126</v>
+      </c>
+      <c r="G8" s="45" t="s">
+        <v>124</v>
+      </c>
+      <c r="H8" s="45">
         <v>350</v>
       </c>
-      <c r="I8" s="47" t="s">
+      <c r="I8" s="46" t="s">
         <v>15</v>
       </c>
-      <c r="J8" s="47">
+      <c r="J8" s="46">
         <v>1</v>
       </c>
       <c r="K8" s="2"/>
       <c r="L8" s="14"/>
-      <c r="O8" s="46"/>
+      <c r="O8" s="45"/>
     </row>
     <row r="9" spans="2:15" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B9" s="12">
@@ -1893,29 +1895,29 @@
         <v>4</v>
       </c>
       <c r="D9" s="13" t="s">
+        <v>117</v>
+      </c>
+      <c r="E9" s="45" t="s">
+        <v>12</v>
+      </c>
+      <c r="F9" s="45" t="s">
+        <v>126</v>
+      </c>
+      <c r="G9" s="45" t="s">
+        <v>124</v>
+      </c>
+      <c r="H9" s="45">
+        <v>1743</v>
+      </c>
+      <c r="I9" s="46" t="s">
+        <v>17</v>
+      </c>
+      <c r="J9" s="46" t="s">
         <v>118</v>
-      </c>
-      <c r="E9" s="46" t="s">
-        <v>12</v>
-      </c>
-      <c r="F9" s="46" t="s">
-        <v>127</v>
-      </c>
-      <c r="G9" s="46" t="s">
-        <v>125</v>
-      </c>
-      <c r="H9" s="46">
-        <v>1743</v>
-      </c>
-      <c r="I9" s="47" t="s">
-        <v>17</v>
-      </c>
-      <c r="J9" s="47" t="s">
-        <v>119</v>
       </c>
       <c r="K9" s="2"/>
       <c r="L9" s="14"/>
-      <c r="O9" s="46"/>
+      <c r="O9" s="45"/>
     </row>
     <row r="10" spans="2:15" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B10" s="12">
@@ -1925,25 +1927,29 @@
         <v>6</v>
       </c>
       <c r="D10" s="13" t="s">
-        <v>40</v>
-      </c>
-      <c r="E10" s="46" t="s">
+        <v>39</v>
+      </c>
+      <c r="E10" s="45" t="s">
         <v>12</v>
       </c>
-      <c r="F10" s="46" t="s">
-        <v>127</v>
-      </c>
-      <c r="G10" s="46" t="s">
-        <v>125</v>
-      </c>
-      <c r="H10" s="46"/>
-      <c r="I10" s="47" t="s">
+      <c r="F10" s="45" t="s">
+        <v>126</v>
+      </c>
+      <c r="G10" s="45" t="s">
+        <v>124</v>
+      </c>
+      <c r="H10" s="45">
+        <v>339</v>
+      </c>
+      <c r="I10" s="46" t="s">
         <v>18</v>
       </c>
-      <c r="J10" s="47"/>
+      <c r="J10" s="46">
+        <v>0</v>
+      </c>
       <c r="K10" s="2"/>
       <c r="L10" s="14"/>
-      <c r="O10" s="46"/>
+      <c r="O10" s="45"/>
     </row>
     <row r="11" spans="2:15" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B11" s="12">
@@ -1953,25 +1959,29 @@
         <v>5</v>
       </c>
       <c r="D11" s="13" t="s">
-        <v>39</v>
-      </c>
-      <c r="E11" s="46" t="s">
+        <v>38</v>
+      </c>
+      <c r="E11" s="45" t="s">
         <v>12</v>
       </c>
-      <c r="F11" s="46" t="s">
-        <v>127</v>
-      </c>
-      <c r="G11" s="46" t="s">
-        <v>125</v>
-      </c>
-      <c r="H11" s="46"/>
-      <c r="I11" s="47" t="s">
+      <c r="F11" s="45" t="s">
+        <v>126</v>
+      </c>
+      <c r="G11" s="45" t="s">
+        <v>124</v>
+      </c>
+      <c r="H11" s="45">
+        <v>109</v>
+      </c>
+      <c r="I11" s="46" t="s">
         <v>18</v>
       </c>
-      <c r="J11" s="47"/>
+      <c r="J11" s="46">
+        <v>2</v>
+      </c>
       <c r="K11" s="2"/>
       <c r="L11" s="14"/>
-      <c r="O11" s="46"/>
+      <c r="O11" s="45"/>
     </row>
     <row r="12" spans="2:15" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B12" s="12">
@@ -1981,27 +1991,27 @@
         <v>5</v>
       </c>
       <c r="D12" s="13" t="s">
-        <v>38</v>
-      </c>
-      <c r="E12" s="46" t="s">
+        <v>37</v>
+      </c>
+      <c r="E12" s="45" t="s">
         <v>12</v>
       </c>
-      <c r="F12" s="46" t="s">
-        <v>127</v>
-      </c>
-      <c r="G12" s="46" t="s">
-        <v>125</v>
-      </c>
-      <c r="H12" s="46"/>
-      <c r="I12" s="47" t="s">
+      <c r="F12" s="45" t="s">
+        <v>126</v>
+      </c>
+      <c r="G12" s="45" t="s">
+        <v>124</v>
+      </c>
+      <c r="H12" s="45"/>
+      <c r="I12" s="46" t="s">
         <v>18</v>
       </c>
-      <c r="J12" s="47">
+      <c r="J12" s="46">
         <v>4</v>
       </c>
       <c r="K12" s="2"/>
       <c r="L12" s="14"/>
-      <c r="O12" s="46"/>
+      <c r="O12" s="45"/>
     </row>
     <row r="13" spans="2:15" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B13" s="12">
@@ -2011,27 +2021,27 @@
         <v>6</v>
       </c>
       <c r="D13" s="13" t="s">
-        <v>37</v>
-      </c>
-      <c r="E13" s="46" t="s">
+        <v>36</v>
+      </c>
+      <c r="E13" s="45" t="s">
         <v>12</v>
       </c>
-      <c r="F13" s="46" t="s">
-        <v>127</v>
-      </c>
-      <c r="G13" s="46" t="s">
-        <v>125</v>
-      </c>
-      <c r="H13" s="46"/>
-      <c r="I13" s="47" t="s">
+      <c r="F13" s="45" t="s">
+        <v>126</v>
+      </c>
+      <c r="G13" s="45" t="s">
+        <v>124</v>
+      </c>
+      <c r="H13" s="45"/>
+      <c r="I13" s="46" t="s">
         <v>18</v>
       </c>
-      <c r="J13" s="47">
-        <v>9</v>
+      <c r="J13" s="46">
+        <v>11</v>
       </c>
       <c r="K13" s="2"/>
       <c r="L13" s="14"/>
-      <c r="O13" s="46"/>
+      <c r="O13" s="45"/>
     </row>
     <row r="14" spans="2:15" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B14" s="12">
@@ -2041,25 +2051,27 @@
         <v>4</v>
       </c>
       <c r="D14" s="13" t="s">
-        <v>36</v>
-      </c>
-      <c r="E14" s="46" t="s">
+        <v>35</v>
+      </c>
+      <c r="E14" s="45" t="s">
         <v>12</v>
       </c>
-      <c r="F14" s="46" t="s">
-        <v>127</v>
-      </c>
-      <c r="G14" s="46" t="s">
-        <v>125</v>
-      </c>
-      <c r="H14" s="46"/>
-      <c r="I14" s="47" t="s">
+      <c r="F14" s="45" t="s">
+        <v>126</v>
+      </c>
+      <c r="G14" s="45" t="s">
+        <v>124</v>
+      </c>
+      <c r="H14" s="45"/>
+      <c r="I14" s="46" t="s">
         <v>19</v>
       </c>
-      <c r="J14" s="47"/>
+      <c r="J14" s="46">
+        <v>5</v>
+      </c>
       <c r="K14" s="2"/>
       <c r="L14" s="14"/>
-      <c r="O14" s="46"/>
+      <c r="O14" s="45"/>
     </row>
     <row r="15" spans="2:15" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B15" s="12">
@@ -2069,25 +2081,27 @@
         <v>7</v>
       </c>
       <c r="D15" s="13" t="s">
-        <v>35</v>
-      </c>
-      <c r="E15" s="46" t="s">
+        <v>34</v>
+      </c>
+      <c r="E15" s="45" t="s">
         <v>12</v>
       </c>
-      <c r="F15" s="46" t="s">
-        <v>127</v>
-      </c>
-      <c r="G15" s="46" t="s">
-        <v>125</v>
-      </c>
-      <c r="H15" s="46"/>
-      <c r="I15" s="47" t="s">
+      <c r="F15" s="45" t="s">
+        <v>126</v>
+      </c>
+      <c r="G15" s="45" t="s">
+        <v>124</v>
+      </c>
+      <c r="H15" s="45"/>
+      <c r="I15" s="46" t="s">
         <v>19</v>
       </c>
-      <c r="J15" s="47"/>
+      <c r="J15" s="46">
+        <v>4</v>
+      </c>
       <c r="K15" s="2"/>
       <c r="L15" s="14"/>
-      <c r="O15" s="46"/>
+      <c r="O15" s="45"/>
     </row>
   </sheetData>
   <phoneticPr fontId="8" type="noConversion"/>
@@ -2114,26 +2128,26 @@
         <v>0</v>
       </c>
       <c r="C3" s="18" t="s">
+        <v>23</v>
+      </c>
+      <c r="D3" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="D3" s="18" t="s">
+      <c r="E3" s="18" t="s">
+        <v>26</v>
+      </c>
+      <c r="F3" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="G3" s="18" t="s">
+        <v>26</v>
+      </c>
+      <c r="H3" s="18" t="s">
         <v>25</v>
-      </c>
-      <c r="E3" s="18" t="s">
-        <v>27</v>
-      </c>
-      <c r="F3" s="18" t="s">
-        <v>30</v>
-      </c>
-      <c r="G3" s="18" t="s">
-        <v>27</v>
-      </c>
-      <c r="H3" s="18" t="s">
-        <v>26</v>
       </c>
       <c r="I3" s="16"/>
       <c r="J3" s="16" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="L3" s="15"/>
     </row>
@@ -2239,7 +2253,7 @@
     <row r="7" spans="2:12" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
     <row r="9" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B9" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C9">
         <f>SUM(C4:C6)</f>
@@ -2264,7 +2278,7 @@
     </row>
     <row r="12" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B12" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D12">
         <f>C9-D9</f>
@@ -2273,26 +2287,26 @@
     </row>
     <row r="14" spans="2:12" x14ac:dyDescent="0.3">
       <c r="C14" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17" s="21" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B18" t="s">
+        <v>45</v>
+      </c>
+      <c r="C18" t="s">
         <v>46</v>
       </c>
-      <c r="C18" t="s">
+      <c r="D18" t="s">
         <v>47</v>
       </c>
-      <c r="D18" t="s">
+      <c r="E18" t="s">
         <v>48</v>
-      </c>
-      <c r="E18" t="s">
-        <v>49</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.3">
@@ -2342,7 +2356,7 @@
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A22" s="21" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B22" s="21">
         <f>SUM(B19:B21)</f>
@@ -2360,7 +2374,7 @@
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B24">
         <f>1068-755</f>
@@ -2369,7 +2383,7 @@
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B25">
         <f>755-212</f>
@@ -2378,7 +2392,7 @@
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A26" s="21" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B26" s="21">
         <f>B24+B25</f>
@@ -2387,7 +2401,7 @@
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A28" s="21" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B28" s="22">
         <f>B26/B22</f>
@@ -2396,7 +2410,7 @@
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A30" s="21" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B30" s="20">
         <f>AVERAGE(E19:E21)</f>
@@ -2405,7 +2419,7 @@
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B31" s="20">
         <f>MEDIAN(E19:E21)</f>
@@ -2431,9 +2445,9 @@
   </cols>
   <sheetData>
     <row r="3" spans="2:7" ht="26.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="C3" s="45"/>
-      <c r="D3" s="45"/>
-      <c r="E3" s="45"/>
+      <c r="C3" s="47"/>
+      <c r="D3" s="47"/>
+      <c r="E3" s="47"/>
     </row>
     <row r="4" spans="2:7" ht="56.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B4" s="4"/>

</xml_diff>